<commit_message>
feat: add Lalezar headings and scenario vocabulary
</commit_message>
<xml_diff>
--- a/docs/14-operations/templates/Teelle_Game_Review_Template_v1.xlsx
+++ b/docs/14-operations/templates/Teelle_Game_Review_Template_v1.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" r:id="R4ea2eff537b64641"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="2" r:id="R247f74841fab46f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="سناریوها" sheetId="3" r:id="R856817fc18f6468a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" r:id="R68fef5e86f4d4fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="2" r:id="R8219921a0b514b90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="سناریوها" sheetId="3" r:id="R8efa890d26744227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="واژه‌نامه سناریو" sheetId="4" r:id="Re952e3389fa34a3c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -174,9 +175,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GamesReviewTable" displayName="GamesReviewTable" ref="A4:AR29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:AR29"/>
-  <x:tableColumns count="44">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GamesReviewTable" displayName="GamesReviewTable" ref="A4:AS29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:AS29"/>
+  <x:tableColumns count="45">
     <x:tableColumn id="1" name="شناسه"/>
     <x:tableColumn id="2" name="عنوان"/>
     <x:tableColumn id="3" name="بازه سنی"/>
@@ -221,30 +222,46 @@
     <x:tableColumn id="42" name="یادداشت بازبین"/>
     <x:tableColumn id="43" name="نام بازبین"/>
     <x:tableColumn id="44" name="تصمیم نهایی"/>
+    <x:tableColumn id="45" name="سناریوی اصلی"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RankingScenariosTable" displayName="RankingScenariosTable" ref="A4:O16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:O16"/>
-  <x:tableColumns count="15">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RankingScenariosTable" displayName="RankingScenariosTable" ref="A4:R16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:R16"/>
+  <x:tableColumns count="18">
     <x:tableColumn id="1" name="شناسه"/>
     <x:tableColumn id="2" name="سن"/>
-    <x:tableColumn id="3" name="شرایط"/>
-    <x:tableColumn id="4" name="مکان"/>
-    <x:tableColumn id="5" name="زمان"/>
-    <x:tableColumn id="6" name="وسایل"/>
-    <x:tableColumn id="7" name="نامزد ۱"/>
-    <x:tableColumn id="8" name="نامزد ۲"/>
-    <x:tableColumn id="9" name="نامزد ۳"/>
-    <x:tableColumn id="10" name="نامزد ۴"/>
-    <x:tableColumn id="11" name="نامزد ۵"/>
-    <x:tableColumn id="12" name="اولویت اول شما"/>
-    <x:tableColumn id="13" name="اولویت دوم شما"/>
-    <x:tableColumn id="14" name="اولویت سوم شما"/>
-    <x:tableColumn id="15" name="دلیل یا اصلاح پیشنهادی"/>
+    <x:tableColumn id="3" name="حالت کودک"/>
+    <x:tableColumn id="4" name="انرژی همراه"/>
+    <x:tableColumn id="5" name="ترکیب گروه"/>
+    <x:tableColumn id="6" name="مکان"/>
+    <x:tableColumn id="7" name="زمان"/>
+    <x:tableColumn id="8" name="وسیله"/>
+    <x:tableColumn id="9" name="هدف"/>
+    <x:tableColumn id="10" name="نامزد ۱"/>
+    <x:tableColumn id="11" name="نامزد ۲"/>
+    <x:tableColumn id="12" name="نامزد ۳"/>
+    <x:tableColumn id="13" name="نامزد ۴"/>
+    <x:tableColumn id="14" name="نامزد ۵"/>
+    <x:tableColumn id="15" name="اولویت اول شما"/>
+    <x:tableColumn id="16" name="اولویت دوم شما"/>
+    <x:tableColumn id="17" name="اولویت سوم شما"/>
+    <x:tableColumn id="18" name="دلیل یا اصلاح پیشنهادی"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ScenarioVocabularyTable" displayName="ScenarioVocabularyTable" ref="A4:C35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:C35"/>
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="بُعد"/>
+    <x:tableColumn id="2" name="کلیدواژه ثابت"/>
+    <x:tableColumn id="3" name="تعریف ثابت"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -477,7 +494,7 @@
         <x:v>کاری که شما انجام می‌دهید</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="42" customHeight="1">
+    <x:row r="5" ht="52" customHeight="1">
       <x:c r="A5" s="11" t="str">
         <x:v>بازی‌ها</x:v>
       </x:c>
@@ -485,51 +502,83 @@
         <x:v>ستون‌های تأیید متن، منبع، سن، ایمنی و تصویر را برای هر بازی تکمیل کنید.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="42" customHeight="1">
+    <x:row r="6" ht="52" customHeight="1">
       <x:c r="A6" s="11" t="str">
-        <x:v>تصویر</x:v>
+        <x:v>فایل یا نشانی تصویر</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
-        <x:v>نام فایل یا نشانی تصویر، متن جایگزین و نکته برش را وارد کنید. فقط تصویری را تأیید کنید که حق استفاده از آن روشن است.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="42" customHeight="1">
+        <x:v>نام فایل تصویر تحویلی یا نشانی مستقیم منبع را بنویسید؛ مثل cup-tower.webp یا https://example.com/cup-tower.jpg. این ستون خود تصویر را داخل فایل قرار نمی‌دهد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52" customHeight="1">
       <x:c r="A7" s="11" t="str">
+        <x:v>متن جایگزین تصویر</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>توصیف کوتاه و کاربردی برای کاربر نابینا یا زمانی که تصویر باز نمی‌شود؛ مثل «کودک و همراه در حال ساختن برج با لیوان‌های سبک».</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52" customHeight="1">
+      <x:c r="A8" s="11" t="str">
+        <x:v>نکته برش</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>بگویید در برش‌های موبایل و دسکتاپ چه چیزی حتماً داخل کادر بماند؛ مثل «دست‌ها و برج در مرکز بمانند و چهره بریده نشود».</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="11" t="str">
+        <x:v>حق استفاده تصویر</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>فقط تصویری را تأیید کنید که مالکیت یا مجوز استفاده از آن روشن است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52" customHeight="1">
+      <x:c r="A10" s="11" t="str">
         <x:v>تصمیم</x:v>
       </x:c>
-      <x:c r="B7" s="11" t="str">
+      <x:c r="B10" s="11" t="str">
         <x:v>برای هر حوزه یکی از گزینه‌های «تأیید»، «نیاز به اصلاح» یا «رد» را انتخاب کنید.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="11" t="str">
+    <x:row r="11" ht="52" customHeight="1">
+      <x:c r="A11" s="11" t="str">
         <x:v>تصمیم نهایی</x:v>
       </x:c>
-      <x:c r="B8" s="11" t="str">
+      <x:c r="B11" s="11" t="str">
         <x:v>وقتی پنج حوزه را بررسی کردید، نتیجه نهایی ردیف را تعیین کنید.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="42" customHeight="1">
-      <x:c r="A9" s="11" t="str">
+    <x:row r="12" ht="52" customHeight="1">
+      <x:c r="A12" s="11" t="str">
         <x:v>سناریوها</x:v>
       </x:c>
-      <x:c r="B9" s="11" t="str">
-        <x:v>برای هر سناریو اولویت اول تا سوم را از میان نامزدها بنویسید و اگر لازم بود دلیل کوتاه اضافه کنید.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="42" customHeight="1">
-      <x:c r="A10" s="11" t="str">
+      <x:c r="B12" s="11" t="str">
+        <x:v>شرایط هر سناریو فقط با کلیدواژه‌های ثابت شیت «واژه‌نامه سناریو» ثبت می‌شود. برای هر سناریو اولویت اول تا سوم را از میان نامزدها بنویسید.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="52" customHeight="1">
+      <x:c r="A13" s="11" t="str">
+        <x:v>سناریوی اصلی بازی</x:v>
+      </x:c>
+      <x:c r="B13" s="11" t="str">
+        <x:v>در ستون زرد «سناریوی اصلی» فقط یک شناسه ثابت مثل S01 انتخاب کنید؛ تعریف آن شناسه در شیت سناریوها تغییر نمی‌کند.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="52" customHeight="1">
+      <x:c r="A14" s="11" t="str">
         <x:v>بازی تازه</x:v>
       </x:c>
-      <x:c r="B10" s="11" t="str">
+      <x:c r="B14" s="11" t="str">
         <x:v>برای افزودن بازی جدید، یک ردیف تازه با شناسه انگلیسی یکتا و همه ستون‌های ضروری بسازید.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="11" t="str">
+    <x:row r="15" ht="52" customHeight="1">
+      <x:c r="A15" s="11" t="str">
         <x:v>تحویل</x:v>
       </x:c>
-      <x:c r="B11" s="11" t="str">
+      <x:c r="B15" s="11" t="str">
         <x:v>فایل تکمیل‌شده را بدون حذف ستون‌ها برگردانید؛ ورود نهایی از مسیر پنل مدیریت و بازبینی مستقل انجام می‌شود.</x:v>
       </x:c>
     </x:row>
@@ -586,6 +635,7 @@
     <x:col min="42" max="42" width="32" hidden="0" customWidth="1"/>
     <x:col min="43" max="43" width="32" hidden="0" customWidth="1"/>
     <x:col min="44" max="44" width="18" hidden="0" customWidth="1"/>
+    <x:col min="45" max="45" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -635,6 +685,7 @@
       <x:c r="AP1" s="1"/>
       <x:c r="AQ1" s="1"/>
       <x:c r="AR1" s="1"/>
+      <x:c r="AS1" s="1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
@@ -683,6 +734,7 @@
       <x:c r="AP2" s="3"/>
       <x:c r="AQ2" s="3"/>
       <x:c r="AR2" s="3"/>
+      <x:c r="AS2" s="3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="20" t="str">
@@ -816,6 +868,9 @@
       </x:c>
       <x:c r="AR4" s="21" t="str">
         <x:v>تصمیم نهایی</x:v>
+      </x:c>
+      <x:c r="AS4" s="21" t="str">
+        <x:v>سناریوی اصلی</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="68" customHeight="1">
@@ -927,6 +982,7 @@
       <x:c r="AR5" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS5" s="23" t="str"/>
     </x:row>
     <x:row r="6" ht="68" customHeight="1">
       <x:c r="A6" s="22" t="str">
@@ -1037,6 +1093,7 @@
       <x:c r="AR6" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS6" s="23" t="str"/>
     </x:row>
     <x:row r="7" ht="68" customHeight="1">
       <x:c r="A7" s="22" t="str">
@@ -1147,6 +1204,7 @@
       <x:c r="AR7" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS7" s="23" t="str"/>
     </x:row>
     <x:row r="8" ht="68" customHeight="1">
       <x:c r="A8" s="22" t="str">
@@ -1257,6 +1315,7 @@
       <x:c r="AR8" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS8" s="23" t="str"/>
     </x:row>
     <x:row r="9" ht="68" customHeight="1">
       <x:c r="A9" s="22" t="str">
@@ -1367,6 +1426,7 @@
       <x:c r="AR9" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS9" s="23" t="str"/>
     </x:row>
     <x:row r="10" ht="68" customHeight="1">
       <x:c r="A10" s="22" t="str">
@@ -1479,6 +1539,7 @@
       <x:c r="AR10" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS10" s="23" t="str"/>
     </x:row>
     <x:row r="11" ht="68" customHeight="1">
       <x:c r="A11" s="22" t="str">
@@ -1589,6 +1650,7 @@
       <x:c r="AR11" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS11" s="23" t="str"/>
     </x:row>
     <x:row r="12" ht="68" customHeight="1">
       <x:c r="A12" s="22" t="str">
@@ -1699,6 +1761,7 @@
       <x:c r="AR12" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS12" s="23" t="str"/>
     </x:row>
     <x:row r="13" ht="68" customHeight="1">
       <x:c r="A13" s="22" t="str">
@@ -1809,6 +1872,7 @@
       <x:c r="AR13" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS13" s="23" t="str"/>
     </x:row>
     <x:row r="14" ht="68" customHeight="1">
       <x:c r="A14" s="22" t="str">
@@ -1921,6 +1985,7 @@
       <x:c r="AR14" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS14" s="23" t="str"/>
     </x:row>
     <x:row r="15" ht="68" customHeight="1">
       <x:c r="A15" s="22" t="str">
@@ -2031,6 +2096,7 @@
       <x:c r="AR15" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS15" s="23" t="str"/>
     </x:row>
     <x:row r="16" ht="68" customHeight="1">
       <x:c r="A16" s="22" t="str">
@@ -2143,6 +2209,7 @@
       <x:c r="AR16" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS16" s="23" t="str"/>
     </x:row>
     <x:row r="17" ht="68" customHeight="1">
       <x:c r="A17" s="22" t="str">
@@ -2255,6 +2322,7 @@
       <x:c r="AR17" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS17" s="23" t="str"/>
     </x:row>
     <x:row r="18" ht="68" customHeight="1">
       <x:c r="A18" s="22" t="str">
@@ -2365,6 +2433,7 @@
       <x:c r="AR18" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS18" s="23" t="str"/>
     </x:row>
     <x:row r="19" ht="68" customHeight="1">
       <x:c r="A19" s="22" t="str">
@@ -2477,6 +2546,7 @@
       <x:c r="AR19" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS19" s="23" t="str"/>
     </x:row>
     <x:row r="20" ht="68" customHeight="1">
       <x:c r="A20" s="22" t="str">
@@ -2589,6 +2659,7 @@
       <x:c r="AR20" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS20" s="23" t="str"/>
     </x:row>
     <x:row r="21" ht="68" customHeight="1">
       <x:c r="A21" s="22" t="str">
@@ -2699,6 +2770,7 @@
       <x:c r="AR21" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS21" s="23" t="str"/>
     </x:row>
     <x:row r="22" ht="68" customHeight="1">
       <x:c r="A22" s="22" t="str">
@@ -2811,6 +2883,7 @@
       <x:c r="AR22" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS22" s="23" t="str"/>
     </x:row>
     <x:row r="23" ht="68" customHeight="1">
       <x:c r="A23" s="22" t="str">
@@ -2921,6 +2994,7 @@
       <x:c r="AR23" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS23" s="23" t="str"/>
     </x:row>
     <x:row r="24" ht="68" customHeight="1">
       <x:c r="A24" s="22" t="str">
@@ -3033,6 +3107,7 @@
       <x:c r="AR24" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS24" s="23" t="str"/>
     </x:row>
     <x:row r="25" ht="68" customHeight="1">
       <x:c r="A25" s="22" t="str">
@@ -3143,6 +3218,7 @@
       <x:c r="AR25" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS25" s="23" t="str"/>
     </x:row>
     <x:row r="26" ht="68" customHeight="1">
       <x:c r="A26" s="22" t="str">
@@ -3255,6 +3331,7 @@
       <x:c r="AR26" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS26" s="23" t="str"/>
     </x:row>
     <x:row r="27" ht="68" customHeight="1">
       <x:c r="A27" s="22" t="str">
@@ -3367,6 +3444,7 @@
       <x:c r="AR27" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS27" s="23" t="str"/>
     </x:row>
     <x:row r="28" ht="68" customHeight="1">
       <x:c r="A28" s="22" t="str">
@@ -3477,6 +3555,7 @@
       <x:c r="AR28" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS28" s="23" t="str"/>
     </x:row>
     <x:row r="29" ht="68" customHeight="1">
       <x:c r="A29" s="22" t="str">
@@ -3589,19 +3668,23 @@
       <x:c r="AR29" s="23" t="str">
         <x:v>در انتظار</x:v>
       </x:c>
+      <x:c r="AS29" s="23" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="AH5:AL29">
       <x:formula1>"تأیید,نیاز به اصلاح,رد"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="AR5:AR29">
       <x:formula1>"در انتظار,تأیید نهایی,نیاز به اصلاح,رد"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="AS5:AS29">
+      <x:formula1>"S01,S02,S03,S04,S05,S06,S07,S08,S09,S10,S11,S12"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8461c476abd947a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R962d8c5b967b4fbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3612,19 +3695,22 @@
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="27" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="27" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="27" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="42" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="24" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -3645,10 +3731,13 @@
       <x:c r="M1" s="1"/>
       <x:c r="N1" s="1"/>
       <x:c r="O1" s="1"/>
+      <x:c r="P1" s="1"/>
+      <x:c r="Q1" s="1"/>
+      <x:c r="R1" s="1"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>برای هر ردیف سه انتخاب برتر را بنویسید؛ ترتیب شما برای تنظیم Ranking استفاده می‌شود.</x:v>
+        <x:v>شرایط از کلیدواژه‌های ثابت انتخاب می‌شوند؛ سه انتخاب برتر شما برای تنظیم Ranking استفاده می‌شود.</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -3664,6 +3753,9 @@
       <x:c r="M2" s="3"/>
       <x:c r="N2" s="3"/>
       <x:c r="O2" s="3"/>
+      <x:c r="P2" s="3"/>
+      <x:c r="Q2" s="3"/>
+      <x:c r="R2" s="3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="25" t="str">
@@ -3673,42 +3765,51 @@
         <x:v>سن</x:v>
       </x:c>
       <x:c r="C4" s="25" t="str">
-        <x:v>شرایط</x:v>
+        <x:v>حالت کودک</x:v>
       </x:c>
       <x:c r="D4" s="25" t="str">
+        <x:v>انرژی همراه</x:v>
+      </x:c>
+      <x:c r="E4" s="25" t="str">
+        <x:v>ترکیب گروه</x:v>
+      </x:c>
+      <x:c r="F4" s="25" t="str">
         <x:v>مکان</x:v>
       </x:c>
-      <x:c r="E4" s="25" t="str">
+      <x:c r="G4" s="25" t="str">
         <x:v>زمان</x:v>
       </x:c>
-      <x:c r="F4" s="25" t="str">
-        <x:v>وسایل</x:v>
-      </x:c>
-      <x:c r="G4" s="25" t="str">
+      <x:c r="H4" s="25" t="str">
+        <x:v>وسیله</x:v>
+      </x:c>
+      <x:c r="I4" s="25" t="str">
+        <x:v>هدف</x:v>
+      </x:c>
+      <x:c r="J4" s="25" t="str">
         <x:v>نامزد ۱</x:v>
       </x:c>
-      <x:c r="H4" s="25" t="str">
+      <x:c r="K4" s="25" t="str">
         <x:v>نامزد ۲</x:v>
       </x:c>
-      <x:c r="I4" s="25" t="str">
+      <x:c r="L4" s="25" t="str">
         <x:v>نامزد ۳</x:v>
       </x:c>
-      <x:c r="J4" s="25" t="str">
+      <x:c r="M4" s="25" t="str">
         <x:v>نامزد ۴</x:v>
       </x:c>
-      <x:c r="K4" s="25" t="str">
+      <x:c r="N4" s="25" t="str">
         <x:v>نامزد ۵</x:v>
       </x:c>
-      <x:c r="L4" s="26" t="str">
+      <x:c r="O4" s="26" t="str">
         <x:v>اولویت اول شما</x:v>
       </x:c>
-      <x:c r="M4" s="26" t="str">
+      <x:c r="P4" s="26" t="str">
         <x:v>اولویت دوم شما</x:v>
       </x:c>
-      <x:c r="N4" s="26" t="str">
+      <x:c r="Q4" s="26" t="str">
         <x:v>اولویت سوم شما</x:v>
       </x:c>
-      <x:c r="O4" s="26" t="str">
+      <x:c r="R4" s="26" t="str">
         <x:v>دلیل یا اصلاح پیشنهادی</x:v>
       </x:c>
     </x:row>
@@ -3720,36 +3821,45 @@
         <x:v>۹ ماه</x:v>
       </x:c>
       <x:c r="C5" s="22" t="str">
-        <x:v>کودک آرام؛ همراه کم‌انرژی</x:v>
+        <x:v>آرام</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
-        <x:v>خانه، روی زمین یا بغل</x:v>
+        <x:v>کم</x:v>
       </x:c>
       <x:c r="E5" s="22" t="str">
-        <x:v>۵ دقیقه</x:v>
+        <x:v>یک‌کودک</x:v>
       </x:c>
       <x:c r="F5" s="22" t="str">
-        <x:v>بدون وسیله</x:v>
+        <x:v>خانه</x:v>
       </x:c>
       <x:c r="G5" s="22" t="str">
+        <x:v>۵دقیقه</x:v>
+      </x:c>
+      <x:c r="H5" s="22" t="str">
+        <x:v>بدون‌وسیله</x:v>
+      </x:c>
+      <x:c r="I5" s="22" t="str">
+        <x:v>ارتباط</x:v>
+      </x:c>
+      <x:c r="J5" s="22" t="str">
         <x:v>آینه‌ی شکلک‌ها</x:v>
       </x:c>
-      <x:c r="H5" s="22" t="str">
+      <x:c r="K5" s="22" t="str">
         <x:v>آواز و مکث</x:v>
       </x:c>
-      <x:c r="I5" s="22" t="str">
+      <x:c r="L5" s="22" t="str">
         <x:v>تو بگو، من تکرار می‌کنم</x:v>
       </x:c>
-      <x:c r="J5" s="22" t="str">
+      <x:c r="M5" s="22" t="str">
         <x:v>صدا از کجاست</x:v>
       </x:c>
-      <x:c r="K5" s="22" t="str">
+      <x:c r="N5" s="22" t="str">
         <x:v>دنبال دست‌های من</x:v>
       </x:c>
-      <x:c r="L5" s="23" t="str"/>
-      <x:c r="M5" s="23" t="str"/>
-      <x:c r="N5" s="23" t="str"/>
       <x:c r="O5" s="23" t="str"/>
+      <x:c r="P5" s="23" t="str"/>
+      <x:c r="Q5" s="23" t="str"/>
+      <x:c r="R5" s="23" t="str"/>
     </x:row>
     <x:row r="6" ht="55" customHeight="1">
       <x:c r="A6" s="22" t="str">
@@ -3759,36 +3869,45 @@
         <x:v>۱۸ ماه</x:v>
       </x:c>
       <x:c r="C6" s="22" t="str">
-        <x:v>بی‌قراری و نیاز به ارتباط</x:v>
+        <x:v>بی‌قرار</x:v>
       </x:c>
       <x:c r="D6" s="22" t="str">
+        <x:v>متوسط</x:v>
+      </x:c>
+      <x:c r="E6" s="22" t="str">
+        <x:v>یک‌کودک</x:v>
+      </x:c>
+      <x:c r="F6" s="22" t="str">
         <x:v>خانه</x:v>
       </x:c>
-      <x:c r="E6" s="22" t="str">
-        <x:v>۵ تا ۸ دقیقه</x:v>
-      </x:c>
-      <x:c r="F6" s="22" t="str">
-        <x:v>بدون وسیله</x:v>
-      </x:c>
       <x:c r="G6" s="22" t="str">
+        <x:v>۵دقیقه</x:v>
+      </x:c>
+      <x:c r="H6" s="22" t="str">
+        <x:v>بدون‌وسیله</x:v>
+      </x:c>
+      <x:c r="I6" s="22" t="str">
+        <x:v>آرام‌سازی</x:v>
+      </x:c>
+      <x:c r="J6" s="22" t="str">
         <x:v>دنبال دست‌های من</x:v>
       </x:c>
-      <x:c r="H6" s="22" t="str">
+      <x:c r="K6" s="22" t="str">
         <x:v>آواز و مکث</x:v>
       </x:c>
-      <x:c r="I6" s="22" t="str">
+      <x:c r="L6" s="22" t="str">
         <x:v>صدا از کجاست</x:v>
       </x:c>
-      <x:c r="J6" s="22" t="str">
+      <x:c r="M6" s="22" t="str">
         <x:v>آینه‌ی شکلک‌ها</x:v>
       </x:c>
-      <x:c r="K6" s="22" t="str">
+      <x:c r="N6" s="22" t="str">
         <x:v>تو بگو، من تکرار می‌کنم</x:v>
       </x:c>
-      <x:c r="L6" s="23" t="str"/>
-      <x:c r="M6" s="23" t="str"/>
-      <x:c r="N6" s="23" t="str"/>
       <x:c r="O6" s="23" t="str"/>
+      <x:c r="P6" s="23" t="str"/>
+      <x:c r="Q6" s="23" t="str"/>
+      <x:c r="R6" s="23" t="str"/>
     </x:row>
     <x:row r="7" ht="55" customHeight="1">
       <x:c r="A7" s="22" t="str">
@@ -3798,36 +3917,45 @@
         <x:v>۳۰ ماه</x:v>
       </x:c>
       <x:c r="C7" s="22" t="str">
-        <x:v>پرانرژی؛ همراه انرژی متوسط</x:v>
+        <x:v>پرانرژی</x:v>
       </x:c>
       <x:c r="D7" s="22" t="str">
+        <x:v>متوسط</x:v>
+      </x:c>
+      <x:c r="E7" s="22" t="str">
+        <x:v>یک‌کودک</x:v>
+      </x:c>
+      <x:c r="F7" s="22" t="str">
         <x:v>خانه</x:v>
       </x:c>
-      <x:c r="E7" s="22" t="str">
-        <x:v>۱۰ دقیقه</x:v>
-      </x:c>
-      <x:c r="F7" s="22" t="str">
-        <x:v>بدون وسیله</x:v>
-      </x:c>
       <x:c r="G7" s="22" t="str">
+        <x:v>۱۰دقیقه</x:v>
+      </x:c>
+      <x:c r="H7" s="22" t="str">
+        <x:v>بدون‌وسیله</x:v>
+      </x:c>
+      <x:c r="I7" s="22" t="str">
+        <x:v>تخلیه‌انرژی</x:v>
+      </x:c>
+      <x:c r="J7" s="22" t="str">
         <x:v>راه‌رفتن حیوان‌ها</x:v>
       </x:c>
-      <x:c r="H7" s="22" t="str">
+      <x:c r="K7" s="22" t="str">
         <x:v>رنگ را پیدا کن</x:v>
       </x:c>
-      <x:c r="I7" s="22" t="str">
+      <x:c r="L7" s="22" t="str">
         <x:v>برج لیوانی</x:v>
       </x:c>
-      <x:c r="J7" s="22" t="str">
+      <x:c r="M7" s="22" t="str">
         <x:v>قصه‌ی نیمه‌کاره</x:v>
       </x:c>
-      <x:c r="K7" s="22" t="str">
+      <x:c r="N7" s="22" t="str">
         <x:v>جورچین لباس‌ها</x:v>
       </x:c>
-      <x:c r="L7" s="23" t="str"/>
-      <x:c r="M7" s="23" t="str"/>
-      <x:c r="N7" s="23" t="str"/>
       <x:c r="O7" s="23" t="str"/>
+      <x:c r="P7" s="23" t="str"/>
+      <x:c r="Q7" s="23" t="str"/>
+      <x:c r="R7" s="23" t="str"/>
     </x:row>
     <x:row r="8" ht="55" customHeight="1">
       <x:c r="A8" s="22" t="str">
@@ -3837,36 +3965,45 @@
         <x:v>۳ سال</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
-        <x:v>نزدیک خواب؛ بازی آرام</x:v>
+        <x:v>نزدیک‌خواب</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
-        <x:v>خانه یا سفر</x:v>
+        <x:v>کم</x:v>
       </x:c>
       <x:c r="E8" s="22" t="str">
-        <x:v>۱۰ دقیقه</x:v>
+        <x:v>یک‌کودک</x:v>
       </x:c>
       <x:c r="F8" s="22" t="str">
-        <x:v>بدون وسیله</x:v>
+        <x:v>سفر</x:v>
       </x:c>
       <x:c r="G8" s="22" t="str">
+        <x:v>۱۰دقیقه</x:v>
+      </x:c>
+      <x:c r="H8" s="22" t="str">
+        <x:v>بدون‌وسیله</x:v>
+      </x:c>
+      <x:c r="I8" s="22" t="str">
+        <x:v>آرام‌سازی</x:v>
+      </x:c>
+      <x:c r="J8" s="22" t="str">
         <x:v>قصه‌ی نیمه‌کاره</x:v>
       </x:c>
-      <x:c r="H8" s="22" t="str">
+      <x:c r="K8" s="22" t="str">
         <x:v>جورچین لباس‌ها</x:v>
       </x:c>
-      <x:c r="I8" s="22" t="str">
+      <x:c r="L8" s="22" t="str">
         <x:v>رنگ را پیدا کن</x:v>
       </x:c>
-      <x:c r="J8" s="22" t="str">
+      <x:c r="M8" s="22" t="str">
         <x:v>برج لیوانی</x:v>
       </x:c>
-      <x:c r="K8" s="22" t="str">
+      <x:c r="N8" s="22" t="str">
         <x:v>راه‌رفتن حیوان‌ها</x:v>
       </x:c>
-      <x:c r="L8" s="23" t="str"/>
-      <x:c r="M8" s="23" t="str"/>
-      <x:c r="N8" s="23" t="str"/>
       <x:c r="O8" s="23" t="str"/>
+      <x:c r="P8" s="23" t="str"/>
+      <x:c r="Q8" s="23" t="str"/>
+      <x:c r="R8" s="23" t="str"/>
     </x:row>
     <x:row r="9" ht="55" customHeight="1">
       <x:c r="A9" s="22" t="str">
@@ -3876,36 +4013,45 @@
         <x:v>۵ سال</x:v>
       </x:c>
       <x:c r="C9" s="22" t="str">
-        <x:v>پرانرژی و بی‌حوصله</x:v>
+        <x:v>پرانرژی</x:v>
       </x:c>
       <x:c r="D9" s="22" t="str">
+        <x:v>زیاد</x:v>
+      </x:c>
+      <x:c r="E9" s="22" t="str">
+        <x:v>یک‌کودک</x:v>
+      </x:c>
+      <x:c r="F9" s="22" t="str">
         <x:v>خانه</x:v>
       </x:c>
-      <x:c r="E9" s="22" t="str">
-        <x:v>۱۵ دقیقه</x:v>
-      </x:c>
-      <x:c r="F9" s="22" t="str">
-        <x:v>توپ نرم در دسترس</x:v>
-      </x:c>
       <x:c r="G9" s="22" t="str">
+        <x:v>۱۵دقیقه</x:v>
+      </x:c>
+      <x:c r="H9" s="22" t="str">
+        <x:v>توپ‌نرم</x:v>
+      </x:c>
+      <x:c r="I9" s="22" t="str">
+        <x:v>حرکت</x:v>
+      </x:c>
+      <x:c r="J9" s="22" t="str">
         <x:v>مجسمه با دست‌زدن</x:v>
       </x:c>
-      <x:c r="H9" s="22" t="str">
+      <x:c r="K9" s="22" t="str">
         <x:v>دروازه‌ی توپ نرم</x:v>
       </x:c>
-      <x:c r="I9" s="22" t="str">
+      <x:c r="L9" s="22" t="str">
         <x:v>مسیر پتویی</x:v>
       </x:c>
-      <x:c r="J9" s="22" t="str">
+      <x:c r="M9" s="22" t="str">
         <x:v>صدای قصه</x:v>
       </x:c>
-      <x:c r="K9" s="22" t="str">
+      <x:c r="N9" s="22" t="str">
         <x:v>زنجیره‌ی نقاشی</x:v>
       </x:c>
-      <x:c r="L9" s="23" t="str"/>
-      <x:c r="M9" s="23" t="str"/>
-      <x:c r="N9" s="23" t="str"/>
       <x:c r="O9" s="23" t="str"/>
+      <x:c r="P9" s="23" t="str"/>
+      <x:c r="Q9" s="23" t="str"/>
+      <x:c r="R9" s="23" t="str"/>
     </x:row>
     <x:row r="10" ht="55" customHeight="1">
       <x:c r="A10" s="22" t="str">
@@ -3915,36 +4061,45 @@
         <x:v>۶ سال</x:v>
       </x:c>
       <x:c r="C10" s="22" t="str">
-        <x:v>آرام و خلاق؛ همراه کم‌انرژی</x:v>
+        <x:v>آرام</x:v>
       </x:c>
       <x:c r="D10" s="22" t="str">
+        <x:v>کم</x:v>
+      </x:c>
+      <x:c r="E10" s="22" t="str">
+        <x:v>یک‌کودک</x:v>
+      </x:c>
+      <x:c r="F10" s="22" t="str">
         <x:v>خانه</x:v>
       </x:c>
-      <x:c r="E10" s="22" t="str">
-        <x:v>۱۵ دقیقه</x:v>
-      </x:c>
-      <x:c r="F10" s="22" t="str">
-        <x:v>کاغذ و مداد</x:v>
-      </x:c>
       <x:c r="G10" s="22" t="str">
+        <x:v>۱۵دقیقه</x:v>
+      </x:c>
+      <x:c r="H10" s="22" t="str">
+        <x:v>کاغذ-و-مداد</x:v>
+      </x:c>
+      <x:c r="I10" s="22" t="str">
+        <x:v>خلاقیت</x:v>
+      </x:c>
+      <x:c r="J10" s="22" t="str">
         <x:v>زنجیره‌ی نقاشی</x:v>
       </x:c>
-      <x:c r="H10" s="22" t="str">
+      <x:c r="K10" s="22" t="str">
         <x:v>صدای قصه</x:v>
       </x:c>
-      <x:c r="I10" s="22" t="str">
+      <x:c r="L10" s="22" t="str">
         <x:v>دروازه‌ی توپ نرم</x:v>
       </x:c>
-      <x:c r="J10" s="22" t="str">
+      <x:c r="M10" s="22" t="str">
         <x:v>مسیر پتویی</x:v>
       </x:c>
-      <x:c r="K10" s="22" t="str">
+      <x:c r="N10" s="22" t="str">
         <x:v>مجسمه با دست‌زدن</x:v>
       </x:c>
-      <x:c r="L10" s="23" t="str"/>
-      <x:c r="M10" s="23" t="str"/>
-      <x:c r="N10" s="23" t="str"/>
       <x:c r="O10" s="23" t="str"/>
+      <x:c r="P10" s="23" t="str"/>
+      <x:c r="Q10" s="23" t="str"/>
+      <x:c r="R10" s="23" t="str"/>
     </x:row>
     <x:row r="11" ht="55" customHeight="1">
       <x:c r="A11" s="22" t="str">
@@ -3954,36 +4109,45 @@
         <x:v>۸ سال</x:v>
       </x:c>
       <x:c r="C11" s="22" t="str">
-        <x:v>دو کودک؛ بازی کم‌صدا</x:v>
+        <x:v>متعادل</x:v>
       </x:c>
       <x:c r="D11" s="22" t="str">
+        <x:v>متوسط</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="str">
+        <x:v>دوکودک-هم‌سن</x:v>
+      </x:c>
+      <x:c r="F11" s="22" t="str">
         <x:v>خانه</x:v>
       </x:c>
-      <x:c r="E11" s="22" t="str">
-        <x:v>۲۰ دقیقه</x:v>
-      </x:c>
-      <x:c r="F11" s="22" t="str">
-        <x:v>کاغذ</x:v>
-      </x:c>
       <x:c r="G11" s="22" t="str">
+        <x:v>۲۰دقیقه</x:v>
+      </x:c>
+      <x:c r="H11" s="22" t="str">
+        <x:v>کاغذ-و-مداد</x:v>
+      </x:c>
+      <x:c r="I11" s="22" t="str">
+        <x:v>همکاری</x:v>
+      </x:c>
+      <x:c r="J11" s="22" t="str">
         <x:v>داستان زنجیره‌ای</x:v>
       </x:c>
-      <x:c r="H11" s="22" t="str">
+      <x:c r="K11" s="22" t="str">
         <x:v>چالش برج کاغذی</x:v>
       </x:c>
-      <x:c r="I11" s="22" t="str">
+      <x:c r="L11" s="22" t="str">
         <x:v>پانتومیم بی‌صدا</x:v>
       </x:c>
-      <x:c r="J11" s="22" t="str">
+      <x:c r="M11" s="22" t="str">
         <x:v>نقشه‌ی گنج کاغذی</x:v>
       </x:c>
-      <x:c r="K11" s="22" t="str">
+      <x:c r="N11" s="22" t="str">
         <x:v>هدف‌گیری با توپ نرم</x:v>
       </x:c>
-      <x:c r="L11" s="23" t="str"/>
-      <x:c r="M11" s="23" t="str"/>
-      <x:c r="N11" s="23" t="str"/>
       <x:c r="O11" s="23" t="str"/>
+      <x:c r="P11" s="23" t="str"/>
+      <x:c r="Q11" s="23" t="str"/>
+      <x:c r="R11" s="23" t="str"/>
     </x:row>
     <x:row r="12" ht="55" customHeight="1">
       <x:c r="A12" s="22" t="str">
@@ -3993,36 +4157,45 @@
         <x:v>۹ سال</x:v>
       </x:c>
       <x:c r="C12" s="22" t="str">
-        <x:v>فضای باز و انرژی زیاد</x:v>
+        <x:v>پرانرژی</x:v>
       </x:c>
       <x:c r="D12" s="22" t="str">
-        <x:v>پارک</x:v>
+        <x:v>زیاد</x:v>
       </x:c>
       <x:c r="E12" s="22" t="str">
-        <x:v>۲۰ دقیقه</x:v>
+        <x:v>دوکودک-هم‌سن</x:v>
       </x:c>
       <x:c r="F12" s="22" t="str">
-        <x:v>توپ نرم</x:v>
+        <x:v>فضای‌باز</x:v>
       </x:c>
       <x:c r="G12" s="22" t="str">
+        <x:v>۲۰دقیقه</x:v>
+      </x:c>
+      <x:c r="H12" s="22" t="str">
+        <x:v>توپ‌نرم</x:v>
+      </x:c>
+      <x:c r="I12" s="22" t="str">
+        <x:v>تخلیه‌انرژی</x:v>
+      </x:c>
+      <x:c r="J12" s="22" t="str">
         <x:v>هدف‌گیری با توپ نرم</x:v>
       </x:c>
-      <x:c r="H12" s="22" t="str">
+      <x:c r="K12" s="22" t="str">
         <x:v>پانتومیم بی‌صدا</x:v>
       </x:c>
-      <x:c r="I12" s="22" t="str">
+      <x:c r="L12" s="22" t="str">
         <x:v>نقشه‌ی گنج کاغذی</x:v>
       </x:c>
-      <x:c r="J12" s="22" t="str">
+      <x:c r="M12" s="22" t="str">
         <x:v>چالش برج کاغذی</x:v>
       </x:c>
-      <x:c r="K12" s="22" t="str">
+      <x:c r="N12" s="22" t="str">
         <x:v>داستان زنجیره‌ای</x:v>
       </x:c>
-      <x:c r="L12" s="23" t="str"/>
-      <x:c r="M12" s="23" t="str"/>
-      <x:c r="N12" s="23" t="str"/>
       <x:c r="O12" s="23" t="str"/>
+      <x:c r="P12" s="23" t="str"/>
+      <x:c r="Q12" s="23" t="str"/>
+      <x:c r="R12" s="23" t="str"/>
     </x:row>
     <x:row r="13" ht="55" customHeight="1">
       <x:c r="A13" s="22" t="str">
@@ -4032,36 +4205,45 @@
         <x:v>۱۱ سال</x:v>
       </x:c>
       <x:c r="C13" s="22" t="str">
-        <x:v>گفت‌وگو و خنده؛ بدون وسیله</x:v>
+        <x:v>متعادل</x:v>
       </x:c>
       <x:c r="D13" s="22" t="str">
-        <x:v>خانه یا سفر</x:v>
+        <x:v>کم</x:v>
       </x:c>
       <x:c r="E13" s="22" t="str">
-        <x:v>۲۰ دقیقه</x:v>
+        <x:v>یک‌کودک</x:v>
       </x:c>
       <x:c r="F13" s="22" t="str">
-        <x:v>بدون وسیله</x:v>
+        <x:v>سفر</x:v>
       </x:c>
       <x:c r="G13" s="22" t="str">
+        <x:v>۲۰دقیقه</x:v>
+      </x:c>
+      <x:c r="H13" s="22" t="str">
+        <x:v>بدون‌وسیله</x:v>
+      </x:c>
+      <x:c r="I13" s="22" t="str">
+        <x:v>گفت‌وگو</x:v>
+      </x:c>
+      <x:c r="J13" s="22" t="str">
         <x:v>بیست سؤال خانوادگی</x:v>
       </x:c>
-      <x:c r="H13" s="22" t="str">
+      <x:c r="K13" s="22" t="str">
         <x:v>مناظره‌ی خنده‌دار</x:v>
       </x:c>
-      <x:c r="I13" s="22" t="str">
+      <x:c r="L13" s="22" t="str">
         <x:v>مأموریت بی‌صدا</x:v>
       </x:c>
-      <x:c r="J13" s="22" t="str">
+      <x:c r="M13" s="22" t="str">
         <x:v>بازی کاغذی خودمان</x:v>
       </x:c>
-      <x:c r="K13" s="22" t="str">
+      <x:c r="N13" s="22" t="str">
         <x:v>پل کاغذی</x:v>
       </x:c>
-      <x:c r="L13" s="23" t="str"/>
-      <x:c r="M13" s="23" t="str"/>
-      <x:c r="N13" s="23" t="str"/>
       <x:c r="O13" s="23" t="str"/>
+      <x:c r="P13" s="23" t="str"/>
+      <x:c r="Q13" s="23" t="str"/>
+      <x:c r="R13" s="23" t="str"/>
     </x:row>
     <x:row r="14" ht="55" customHeight="1">
       <x:c r="A14" s="22" t="str">
@@ -4071,36 +4253,45 @@
         <x:v>۱۲ سال</x:v>
       </x:c>
       <x:c r="C14" s="22" t="str">
-        <x:v>خلاق و اهل ساختن</x:v>
+        <x:v>آرام</x:v>
       </x:c>
       <x:c r="D14" s="22" t="str">
+        <x:v>متوسط</x:v>
+      </x:c>
+      <x:c r="E14" s="22" t="str">
+        <x:v>یک‌کودک</x:v>
+      </x:c>
+      <x:c r="F14" s="22" t="str">
         <x:v>خانه</x:v>
       </x:c>
-      <x:c r="E14" s="22" t="str">
-        <x:v>۳۰ دقیقه</x:v>
-      </x:c>
-      <x:c r="F14" s="22" t="str">
-        <x:v>کاغذ و لیوان سبک</x:v>
-      </x:c>
       <x:c r="G14" s="22" t="str">
+        <x:v>۳۰دقیقه</x:v>
+      </x:c>
+      <x:c r="H14" s="22" t="str">
+        <x:v>لیوان‌سبک</x:v>
+      </x:c>
+      <x:c r="I14" s="22" t="str">
+        <x:v>خلاقیت</x:v>
+      </x:c>
+      <x:c r="J14" s="22" t="str">
         <x:v>بازی کاغذی خودمان</x:v>
       </x:c>
-      <x:c r="H14" s="22" t="str">
+      <x:c r="K14" s="22" t="str">
         <x:v>پل کاغذی</x:v>
       </x:c>
-      <x:c r="I14" s="22" t="str">
+      <x:c r="L14" s="22" t="str">
         <x:v>مأموریت بی‌صدا</x:v>
       </x:c>
-      <x:c r="J14" s="22" t="str">
+      <x:c r="M14" s="22" t="str">
         <x:v>مناظره‌ی خنده‌دار</x:v>
       </x:c>
-      <x:c r="K14" s="22" t="str">
+      <x:c r="N14" s="22" t="str">
         <x:v>بیست سؤال خانوادگی</x:v>
       </x:c>
-      <x:c r="L14" s="23" t="str"/>
-      <x:c r="M14" s="23" t="str"/>
-      <x:c r="N14" s="23" t="str"/>
       <x:c r="O14" s="23" t="str"/>
+      <x:c r="P14" s="23" t="str"/>
+      <x:c r="Q14" s="23" t="str"/>
+      <x:c r="R14" s="23" t="str"/>
     </x:row>
     <x:row r="15" ht="55" customHeight="1">
       <x:c r="A15" s="22" t="str">
@@ -4110,36 +4301,45 @@
         <x:v>۵ و ۸ سال</x:v>
       </x:c>
       <x:c r="C15" s="22" t="str">
-        <x:v>دو کودک با سن متفاوت</x:v>
+        <x:v>متعادل</x:v>
       </x:c>
       <x:c r="D15" s="22" t="str">
+        <x:v>متوسط</x:v>
+      </x:c>
+      <x:c r="E15" s="22" t="str">
+        <x:v>دوکودک-چندسنی</x:v>
+      </x:c>
+      <x:c r="F15" s="22" t="str">
         <x:v>خانه</x:v>
       </x:c>
-      <x:c r="E15" s="22" t="str">
-        <x:v>۱۵ دقیقه</x:v>
-      </x:c>
-      <x:c r="F15" s="22" t="str">
-        <x:v>توپ نرم یا کاغذ</x:v>
-      </x:c>
       <x:c r="G15" s="22" t="str">
+        <x:v>۱۵دقیقه</x:v>
+      </x:c>
+      <x:c r="H15" s="22" t="str">
+        <x:v>توپ‌نرم</x:v>
+      </x:c>
+      <x:c r="I15" s="22" t="str">
+        <x:v>همکاری</x:v>
+      </x:c>
+      <x:c r="J15" s="22" t="str">
         <x:v>دروازه‌ی توپ نرم</x:v>
       </x:c>
-      <x:c r="H15" s="22" t="str">
+      <x:c r="K15" s="22" t="str">
         <x:v>زنجیره‌ی نقاشی</x:v>
       </x:c>
-      <x:c r="I15" s="22" t="str">
+      <x:c r="L15" s="22" t="str">
         <x:v>داستان زنجیره‌ای</x:v>
       </x:c>
-      <x:c r="J15" s="22" t="str">
+      <x:c r="M15" s="22" t="str">
         <x:v>پانتومیم بی‌صدا</x:v>
       </x:c>
-      <x:c r="K15" s="22" t="str">
+      <x:c r="N15" s="22" t="str">
         <x:v>مجسمه با دست‌زدن</x:v>
       </x:c>
-      <x:c r="L15" s="23" t="str"/>
-      <x:c r="M15" s="23" t="str"/>
-      <x:c r="N15" s="23" t="str"/>
       <x:c r="O15" s="23" t="str"/>
+      <x:c r="P15" s="23" t="str"/>
+      <x:c r="Q15" s="23" t="str"/>
+      <x:c r="R15" s="23" t="str"/>
     </x:row>
     <x:row r="16" ht="55" customHeight="1">
       <x:c r="A16" s="22" t="str">
@@ -4149,41 +4349,456 @@
         <x:v>۳ و ۶ سال</x:v>
       </x:c>
       <x:c r="C16" s="22" t="str">
-        <x:v>دو کودک؛ همراه کم‌انرژی</x:v>
+        <x:v>متعادل</x:v>
       </x:c>
       <x:c r="D16" s="22" t="str">
+        <x:v>کم</x:v>
+      </x:c>
+      <x:c r="E16" s="22" t="str">
+        <x:v>دوکودک-چندسنی</x:v>
+      </x:c>
+      <x:c r="F16" s="22" t="str">
         <x:v>خانه</x:v>
       </x:c>
-      <x:c r="E16" s="22" t="str">
-        <x:v>۱۰ دقیقه</x:v>
-      </x:c>
-      <x:c r="F16" s="22" t="str">
-        <x:v>بدون وسیله</x:v>
-      </x:c>
       <x:c r="G16" s="22" t="str">
+        <x:v>۱۰دقیقه</x:v>
+      </x:c>
+      <x:c r="H16" s="22" t="str">
+        <x:v>بدون‌وسیله</x:v>
+      </x:c>
+      <x:c r="I16" s="22" t="str">
+        <x:v>ارتباط</x:v>
+      </x:c>
+      <x:c r="J16" s="22" t="str">
         <x:v>رنگ را پیدا کن</x:v>
       </x:c>
-      <x:c r="H16" s="22" t="str">
+      <x:c r="K16" s="22" t="str">
         <x:v>قصه‌ی نیمه‌کاره</x:v>
       </x:c>
-      <x:c r="I16" s="22" t="str">
+      <x:c r="L16" s="22" t="str">
         <x:v>صدای قصه</x:v>
       </x:c>
-      <x:c r="J16" s="22" t="str">
+      <x:c r="M16" s="22" t="str">
         <x:v>مجسمه با دست‌زدن</x:v>
       </x:c>
-      <x:c r="K16" s="22" t="str">
+      <x:c r="N16" s="22" t="str">
         <x:v>برج لیوانی</x:v>
       </x:c>
-      <x:c r="L16" s="23" t="str"/>
-      <x:c r="M16" s="23" t="str"/>
-      <x:c r="N16" s="23" t="str"/>
       <x:c r="O16" s="23" t="str"/>
+      <x:c r="P16" s="23" t="str"/>
+      <x:c r="Q16" s="23" t="str"/>
+      <x:c r="R16" s="23" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="7">
+    <x:dataValidation type="list" sqref="C5:C16">
+      <x:formula1>"آرام,متعادل,پرانرژی,بی‌قرار,نزدیک‌خواب"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D5:D16">
+      <x:formula1>"کم,متوسط,زیاد"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E5:E16">
+      <x:formula1>"یک‌کودک,دوکودک-هم‌سن,دوکودک-چندسنی"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F5:F16">
+      <x:formula1>"خانه,فضای‌باز,سفر"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G5:G16">
+      <x:formula1>"۵دقیقه,۱۰دقیقه,۱۵دقیقه,۲۰دقیقه,۳۰دقیقه"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="H5:H16">
+      <x:formula1>"بدون‌وسیله,کاغذ-و-مداد,توپ‌نرم,پتو,لیوان‌سبک"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I5:I16">
+      <x:formula1>"ارتباط,آرام‌سازی,تخلیه‌انرژی,خلاقیت,گفت‌وگو,همکاری,حرکت"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re01bfea7cbbb4b23"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="68" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>واژه‌نامه ثابت سناریوها</x:v>
+      </x:c>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="3" t="str">
+        <x:v>فقط همین کلیدواژه‌ها در سناریوها استفاده می‌شوند؛ هر تغییر در تعریف نیازمند نسخه تازه فایل است.</x:v>
+      </x:c>
+      <x:c r="B2" s="3"/>
+      <x:c r="C2" s="3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="25" t="str">
+        <x:v>بُعد</x:v>
+      </x:c>
+      <x:c r="B4" s="25" t="str">
+        <x:v>کلیدواژه ثابت</x:v>
+      </x:c>
+      <x:c r="C4" s="25" t="str">
+        <x:v>تعریف ثابت</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
+      <x:c r="A5" s="22" t="str">
+        <x:v>حالت کودک</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>آرام</x:v>
+      </x:c>
+      <x:c r="C5" s="22" t="str">
+        <x:v>کودک آماده فعالیت کم‌تحرک و متمرکز است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="38" customHeight="1">
+      <x:c r="A6" s="22" t="str">
+        <x:v>حالت کودک</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>متعادل</x:v>
+      </x:c>
+      <x:c r="C6" s="22" t="str">
+        <x:v>سطح انرژی کودک معمولی است و محدودیت برجسته‌ای ندارد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="38" customHeight="1">
+      <x:c r="A7" s="22" t="str">
+        <x:v>حالت کودک</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>پرانرژی</x:v>
+      </x:c>
+      <x:c r="C7" s="22" t="str">
+        <x:v>کودک به فعالیت بدنی و تخلیه انرژی نیاز دارد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="38" customHeight="1">
+      <x:c r="A8" s="22" t="str">
+        <x:v>حالت کودک</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>بی‌قرار</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>کودک تمرکز کوتاه دارد و ابتدا به تنظیم هیجان نیاز دارد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="38" customHeight="1">
+      <x:c r="A9" s="22" t="str">
+        <x:v>حالت کودک</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>نزدیک‌خواب</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>فعالیت باید آرام، کوتاه و بدون برانگیختگی زیاد باشد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="38" customHeight="1">
+      <x:c r="A10" s="22" t="str">
+        <x:v>انرژی همراه</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>کم</x:v>
+      </x:c>
+      <x:c r="C10" s="22" t="str">
+        <x:v>همراه توان اجرای بازی نشسته یا با حرکت کم را دارد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
+      <x:c r="A11" s="22" t="str">
+        <x:v>انرژی همراه</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>متوسط</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
+        <x:v>همراه می‌تواند هدایت و مشارکت معمول داشته باشد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="38" customHeight="1">
+      <x:c r="A12" s="22" t="str">
+        <x:v>انرژی همراه</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>زیاد</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>همراه آماده مشارکت فعال و پرتحرک است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="38" customHeight="1">
+      <x:c r="A13" s="22" t="str">
+        <x:v>ترکیب گروه</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>یک‌کودک</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>یک کودک همراه یک یا چند بزرگسال بازی می‌کند.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="38" customHeight="1">
+      <x:c r="A14" s="22" t="str">
+        <x:v>ترکیب گروه</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>دوکودک-هم‌سن</x:v>
+      </x:c>
+      <x:c r="C14" s="22" t="str">
+        <x:v>دو کودک در یک بازه سنی نزدیک بازی می‌کنند.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="38" customHeight="1">
+      <x:c r="A15" s="22" t="str">
+        <x:v>ترکیب گروه</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>دوکودک-چندسنی</x:v>
+      </x:c>
+      <x:c r="C15" s="22" t="str">
+        <x:v>دو کودک با فاصله سنی معنادار بازی می‌کنند.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="38" customHeight="1">
+      <x:c r="A16" s="22" t="str">
+        <x:v>مکان</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>خانه</x:v>
+      </x:c>
+      <x:c r="C16" s="22" t="str">
+        <x:v>بازی در فضای داخلی خانه قابل اجراست.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="38" customHeight="1">
+      <x:c r="A17" s="22" t="str">
+        <x:v>مکان</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>فضای‌باز</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>بازی به حیاط، پارک یا محیط باز مناسب نیاز دارد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="38" customHeight="1">
+      <x:c r="A18" s="22" t="str">
+        <x:v>مکان</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>سفر</x:v>
+      </x:c>
+      <x:c r="C18" s="22" t="str">
+        <x:v>بازی در مسیر یا اقامت سفر با فضای محدود قابل اجراست.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="38" customHeight="1">
+      <x:c r="A19" s="22" t="str">
+        <x:v>زمان</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>۵دقیقه</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>زمان هدف اجرای بازی حدود پنج دقیقه است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="38" customHeight="1">
+      <x:c r="A20" s="22" t="str">
+        <x:v>زمان</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>۱۰دقیقه</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="str">
+        <x:v>زمان هدف اجرای بازی حدود ده دقیقه است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="38" customHeight="1">
+      <x:c r="A21" s="22" t="str">
+        <x:v>زمان</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>۱۵دقیقه</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="str">
+        <x:v>زمان هدف اجرای بازی حدود پانزده دقیقه است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="38" customHeight="1">
+      <x:c r="A22" s="22" t="str">
+        <x:v>زمان</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>۲۰دقیقه</x:v>
+      </x:c>
+      <x:c r="C22" s="22" t="str">
+        <x:v>زمان هدف اجرای بازی حدود بیست دقیقه است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="38" customHeight="1">
+      <x:c r="A23" s="22" t="str">
+        <x:v>زمان</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>۳۰دقیقه</x:v>
+      </x:c>
+      <x:c r="C23" s="22" t="str">
+        <x:v>زمان هدف اجرای بازی حدود سی دقیقه است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="38" customHeight="1">
+      <x:c r="A24" s="22" t="str">
+        <x:v>وسیله</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>بدون‌وسیله</x:v>
+      </x:c>
+      <x:c r="C24" s="22" t="str">
+        <x:v>هیچ وسیله آماده‌سازی‌شده‌ای لازم نیست.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="38" customHeight="1">
+      <x:c r="A25" s="22" t="str">
+        <x:v>وسیله</x:v>
+      </x:c>
+      <x:c r="B25" s="22" t="str">
+        <x:v>کاغذ-و-مداد</x:v>
+      </x:c>
+      <x:c r="C25" s="22" t="str">
+        <x:v>کاغذ و ابزار نوشتن یا نقاشی لازم است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="38" customHeight="1">
+      <x:c r="A26" s="22" t="str">
+        <x:v>وسیله</x:v>
+      </x:c>
+      <x:c r="B26" s="22" t="str">
+        <x:v>توپ‌نرم</x:v>
+      </x:c>
+      <x:c r="C26" s="22" t="str">
+        <x:v>توپ سبک و نرم متناسب با محیط لازم است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="38" customHeight="1">
+      <x:c r="A27" s="22" t="str">
+        <x:v>وسیله</x:v>
+      </x:c>
+      <x:c r="B27" s="22" t="str">
+        <x:v>پتو</x:v>
+      </x:c>
+      <x:c r="C27" s="22" t="str">
+        <x:v>یک پتو یا پارچه بزرگ و امن لازم است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="38" customHeight="1">
+      <x:c r="A28" s="22" t="str">
+        <x:v>وسیله</x:v>
+      </x:c>
+      <x:c r="B28" s="22" t="str">
+        <x:v>لیوان‌سبک</x:v>
+      </x:c>
+      <x:c r="C28" s="22" t="str">
+        <x:v>لیوان سبک و نشکن لازم است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="38" customHeight="1">
+      <x:c r="A29" s="22" t="str">
+        <x:v>هدف</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
+        <x:v>ارتباط</x:v>
+      </x:c>
+      <x:c r="C29" s="22" t="str">
+        <x:v>تمرکز اصلی بازی ایجاد تماس و تعامل میان کودک و همراه است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="38" customHeight="1">
+      <x:c r="A30" s="22" t="str">
+        <x:v>هدف</x:v>
+      </x:c>
+      <x:c r="B30" s="22" t="str">
+        <x:v>آرام‌سازی</x:v>
+      </x:c>
+      <x:c r="C30" s="22" t="str">
+        <x:v>تمرکز اصلی کاهش برانگیختگی و رسیدن به آرامش است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="38" customHeight="1">
+      <x:c r="A31" s="22" t="str">
+        <x:v>هدف</x:v>
+      </x:c>
+      <x:c r="B31" s="22" t="str">
+        <x:v>تخلیه‌انرژی</x:v>
+      </x:c>
+      <x:c r="C31" s="22" t="str">
+        <x:v>تمرکز اصلی مصرف امن انرژی بدنی کودک است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="38" customHeight="1">
+      <x:c r="A32" s="22" t="str">
+        <x:v>هدف</x:v>
+      </x:c>
+      <x:c r="B32" s="22" t="str">
+        <x:v>خلاقیت</x:v>
+      </x:c>
+      <x:c r="C32" s="22" t="str">
+        <x:v>تمرکز اصلی ساختن، خیال‌پردازی یا خلق پاسخ تازه است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="38" customHeight="1">
+      <x:c r="A33" s="22" t="str">
+        <x:v>هدف</x:v>
+      </x:c>
+      <x:c r="B33" s="22" t="str">
+        <x:v>گفت‌وگو</x:v>
+      </x:c>
+      <x:c r="C33" s="22" t="str">
+        <x:v>تمرکز اصلی صحبت، شنیدن و شناخت بیشتر یکدیگر است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="38" customHeight="1">
+      <x:c r="A34" s="22" t="str">
+        <x:v>هدف</x:v>
+      </x:c>
+      <x:c r="B34" s="22" t="str">
+        <x:v>همکاری</x:v>
+      </x:c>
+      <x:c r="C34" s="22" t="str">
+        <x:v>تمرکز اصلی رسیدن مشترک به یک نتیجه است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="38" customHeight="1">
+      <x:c r="A35" s="22" t="str">
+        <x:v>هدف</x:v>
+      </x:c>
+      <x:c r="B35" s="22" t="str">
+        <x:v>حرکت</x:v>
+      </x:c>
+      <x:c r="C35" s="22" t="str">
+        <x:v>تمرکز اصلی حرکت هماهنگ و فعالیت بدنی است.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R987acdaf48294462"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf2e3ca6da184092"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: make phase 14 review workbook usable
</commit_message>
<xml_diff>
--- a/docs/14-operations/templates/Teelle_Game_Review_Template_v1.xlsx
+++ b/docs/14-operations/templates/Teelle_Game_Review_Template_v1.xlsx
@@ -2,10 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" r:id="R68fef5e86f4d4fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="2" r:id="R8219921a0b514b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="سناریوها" sheetId="3" r:id="R8efa890d26744227"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="واژه‌نامه سناریو" sheetId="4" r:id="Re952e3389fa34a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما" sheetId="1" r:id="R38a2cdb23dc54caa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازبینی ساده" sheetId="2" r:id="R00f55023ec8043f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="بازی‌ها" sheetId="3" r:id="Raf18510e86134aa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="سناریوها" sheetId="4" r:id="R019d1d2389fd4894"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="واژه‌نامه سناریو" sheetId="5" r:id="R4729e0d489114255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="مرجع سبک تصویر" sheetId="6" r:id="Re24b24b817f84828"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,7 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -55,8 +57,14 @@
       <x:color rgb="FF123F46"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF123F46"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,6 +84,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFC51632"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE9AD"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -103,7 +116,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -167,6 +180,11 @@
     <x:xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -174,8 +192,64 @@
 </x:styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="10287000" cy="6858000"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="89825edd-f959-43ed-a0b9-0a9994e8a58c"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R98892b86722d4627"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GamesReviewTable" displayName="GamesReviewTable" ref="A4:AS29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SimpleGameReviewTable" displayName="SimpleGameReviewTable" ref="A4:O29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:O29"/>
+  <x:tableColumns count="15">
+    <x:tableColumn id="1" name="پیش‌نمایش تصویر"/>
+    <x:tableColumn id="2" name="عنوان فعلی"/>
+    <x:tableColumn id="3" name="عنوان پیشنهادی شما"/>
+    <x:tableColumn id="4" name="توضیح فعلی"/>
+    <x:tableColumn id="5" name="توضیح پیشنهادی شما"/>
+    <x:tableColumn id="6" name="روش بازی فعلی"/>
+    <x:tableColumn id="7" name="روش پیشنهادی شما"/>
+    <x:tableColumn id="8" name="نکته ایمنی فعلی"/>
+    <x:tableColumn id="9" name="ایمنی پیشنهادی شما"/>
+    <x:tableColumn id="10" name="تصمیم متن"/>
+    <x:tableColumn id="11" name="تصمیم تصویر"/>
+    <x:tableColumn id="12" name="فایل یا نشانی تصویر"/>
+    <x:tableColumn id="13" name="متن جایگزین تصویر"/>
+    <x:tableColumn id="14" name="نکته برش"/>
+    <x:tableColumn id="15" name="یادداشت شما"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GamesReviewTable" displayName="GamesReviewTable" ref="A4:AS29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:AS29"/>
   <x:tableColumns count="45">
     <x:tableColumn id="1" name="شناسه"/>
@@ -228,8 +302,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RankingScenariosTable" displayName="RankingScenariosTable" ref="A4:R16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RankingScenariosTable" displayName="RankingScenariosTable" ref="A4:R16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:R16"/>
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="شناسه"/>
@@ -255,8 +329,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ScenarioVocabularyTable" displayName="ScenarioVocabularyTable" ref="A4:C35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ScenarioVocabularyTable" displayName="ScenarioVocabularyTable" ref="A4:C35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A4:C35"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="بُعد"/>
@@ -478,7 +552,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>نسخه ۱ — فهرست پیشنهادی ۲۵ بازی و ورودی موردنیاز برای انتشار</x:v>
+        <x:v>از شیت «بازبینی ساده» شروع کنید؛ متن فعلی می‌ماند و پیشنهاد شما در ستون زرد نوشته می‌شود</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -491,95 +565,111 @@
         <x:v>بخش</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str">
-        <x:v>کاری که شما انجام می‌دهید</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="52" customHeight="1">
+        <x:v>چه کار کنم؟</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="58" customHeight="1">
       <x:c r="A5" s="11" t="str">
-        <x:v>بازی‌ها</x:v>
+        <x:v>از کجا شروع کنم؟</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>ستون‌های تأیید متن، منبع، سن، ایمنی و تصویر را برای هر بازی تکمیل کنید.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="52" customHeight="1">
+        <x:v>شیت «بازبینی ساده» را باز کنید. هر بازی یک ردیف دارد و چیزهایی که باید بررسی کنید کنار هم هستند.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="58" customHeight="1">
       <x:c r="A6" s="11" t="str">
+        <x:v>عنوان بازی</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>اگر عنوان فعلی خوب است، ستون زرد «عنوان پیشنهادی شما» را خالی بگذارید. اگر تغییر می‌خواهید، عنوان تازه را همان‌جا بنویسید.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="58" customHeight="1">
+      <x:c r="A7" s="11" t="str">
+        <x:v>توضیح کوتاه</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>نسخه پیشنهادی خودتان را در ستون زرد «توضیح پیشنهادی شما» بنویسید. متن فعلی پاک نمی‌شود و کنار آن می‌ماند.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="58" customHeight="1">
+      <x:c r="A8" s="11" t="str">
+        <x:v>روش بازی</x:v>
+      </x:c>
+      <x:c r="B8" s="11" t="str">
+        <x:v>اگر مراحل نیاز به تغییر دارند، نسخه کامل و نهایی را در ستون زرد «روش پیشنهادی شما» بنویسید. مرحله‌ها را با | از هم جدا کنید.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="58" customHeight="1">
+      <x:c r="A9" s="11" t="str">
+        <x:v>نکته ایمنی</x:v>
+      </x:c>
+      <x:c r="B9" s="11" t="str">
+        <x:v>اگر متن ایمنی نیاز به اصلاح دارد، نسخه کامل پیشنهادی را در ستون زرد «ایمنی پیشنهادی شما» بنویسید.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="58" customHeight="1">
+      <x:c r="A10" s="11" t="str">
+        <x:v>پیش‌نمایش تصویر</x:v>
+      </x:c>
+      <x:c r="B10" s="11" t="str">
+        <x:v>تصویر پیشنهادی باید در ستون اول همان ردیف دیده شود. اگر نوشته «هنوز تصویر پیشنهادی نداریم»، آن بازی فعلاً تصویر قابل تأیید ندارد.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
+      <x:c r="A11" s="11" t="str">
+        <x:v>تصمیم متن</x:v>
+      </x:c>
+      <x:c r="B11" s="11" t="str">
+        <x:v>بعد از خواندن متن و نوشتن اصلاحات، یکی از گزینه‌های «تأیید»، «نیاز به اصلاح» یا «رد» را انتخاب کنید.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="11" t="str">
+        <x:v>تصمیم تصویر</x:v>
+      </x:c>
+      <x:c r="B12" s="11" t="str">
+        <x:v>فقط وقتی تصویر را واقعاً می‌بینید تأیید یا رد کنید. تا قبل از آن گزینه «در انتظار تصویر» باید باقی بماند.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58" customHeight="1">
+      <x:c r="A13" s="11" t="str">
         <x:v>فایل یا نشانی تصویر</x:v>
       </x:c>
-      <x:c r="B6" s="11" t="str">
-        <x:v>نام فایل تصویر تحویلی یا نشانی مستقیم منبع را بنویسید؛ مثل cup-tower.webp یا https://example.com/cup-tower.jpg. این ستون خود تصویر را داخل فایل قرار نمی‌دهد.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="52" customHeight="1">
-      <x:c r="A7" s="11" t="str">
+      <x:c r="B13" s="11" t="str">
+        <x:v>نام فایل تحویلی یا نشانی مستقیم منبع را وارد کنید؛ مثل cup-tower.png یا https://example.com/cup-tower.jpg.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="58" customHeight="1">
+      <x:c r="A14" s="11" t="str">
         <x:v>متن جایگزین تصویر</x:v>
       </x:c>
-      <x:c r="B7" s="11" t="str">
-        <x:v>توصیف کوتاه و کاربردی برای کاربر نابینا یا زمانی که تصویر باز نمی‌شود؛ مثل «کودک و همراه در حال ساختن برج با لیوان‌های سبک».</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="52" customHeight="1">
-      <x:c r="A8" s="11" t="str">
+      <x:c r="B14" s="11" t="str">
+        <x:v>خیلی کوتاه بگویید در تصویر چه اتفاقی می‌افتد؛ مثل «کودک و همراه در حال ساختن برج با لیوان‌های سبک».</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="58" customHeight="1">
+      <x:c r="A15" s="11" t="str">
         <x:v>نکته برش</x:v>
       </x:c>
-      <x:c r="B8" s="11" t="str">
-        <x:v>بگویید در برش‌های موبایل و دسکتاپ چه چیزی حتماً داخل کادر بماند؛ مثل «دست‌ها و برج در مرکز بمانند و چهره بریده نشود».</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="52" customHeight="1">
-      <x:c r="A9" s="11" t="str">
-        <x:v>حق استفاده تصویر</x:v>
-      </x:c>
-      <x:c r="B9" s="11" t="str">
-        <x:v>فقط تصویری را تأیید کنید که مالکیت یا مجوز استفاده از آن روشن است.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="52" customHeight="1">
-      <x:c r="A10" s="11" t="str">
-        <x:v>تصمیم</x:v>
-      </x:c>
-      <x:c r="B10" s="11" t="str">
-        <x:v>برای هر حوزه یکی از گزینه‌های «تأیید»، «نیاز به اصلاح» یا «رد» را انتخاب کنید.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="52" customHeight="1">
-      <x:c r="A11" s="11" t="str">
-        <x:v>تصمیم نهایی</x:v>
-      </x:c>
-      <x:c r="B11" s="11" t="str">
-        <x:v>وقتی پنج حوزه را بررسی کردید، نتیجه نهایی ردیف را تعیین کنید.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="52" customHeight="1">
-      <x:c r="A12" s="11" t="str">
+      <x:c r="B15" s="11" t="str">
+        <x:v>بگویید در نسخه موبایل و دسکتاپ چه چیزی حتماً داخل کادر بماند؛ مثل «دست‌ها و برج در مرکز بمانند».</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="58" customHeight="1">
+      <x:c r="A16" s="11" t="str">
         <x:v>سناریوها</x:v>
       </x:c>
-      <x:c r="B12" s="11" t="str">
-        <x:v>شرایط هر سناریو فقط با کلیدواژه‌های ثابت شیت «واژه‌نامه سناریو» ثبت می‌شود. برای هر سناریو اولویت اول تا سوم را از میان نامزدها بنویسید.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="52" customHeight="1">
-      <x:c r="A13" s="11" t="str">
-        <x:v>سناریوی اصلی بازی</x:v>
-      </x:c>
-      <x:c r="B13" s="11" t="str">
-        <x:v>در ستون زرد «سناریوی اصلی» فقط یک شناسه ثابت مثل S01 انتخاب کنید؛ تعریف آن شناسه در شیت سناریوها تغییر نمی‌کند.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="52" customHeight="1">
-      <x:c r="A14" s="11" t="str">
-        <x:v>بازی تازه</x:v>
-      </x:c>
-      <x:c r="B14" s="11" t="str">
-        <x:v>برای افزودن بازی جدید، یک ردیف تازه با شناسه انگلیسی یکتا و همه ستون‌های ضروری بسازید.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="52" customHeight="1">
-      <x:c r="A15" s="11" t="str">
-        <x:v>تحویل</x:v>
-      </x:c>
-      <x:c r="B15" s="11" t="str">
-        <x:v>فایل تکمیل‌شده را بدون حذف ستون‌ها برگردانید؛ ورود نهایی از مسیر پنل مدیریت و بازبینی مستقل انجام می‌شود.</x:v>
+      <x:c r="B16" s="11" t="str">
+        <x:v>در شیت «سناریوها» سه بازی برتر هر موقعیت را انتخاب کنید. معنی کلیدواژه‌ها در شیت «واژه‌نامه سناریو» ثابت شده است.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="11" t="str">
+        <x:v>تحویل فایل</x:v>
+      </x:c>
+      <x:c r="B17" s="11" t="str">
+        <x:v>فایل را بدون حذف ستون‌ها برگردانید. خانه‌های زرد ورودی شما هستند و خانه‌های سفید نسخه فعلی را نشان می‌دهند.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -588,6 +678,853 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="38" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="30" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>بازبینی ساده بازی‌ها</x:v>
+      </x:c>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+      <x:c r="K1" s="1"/>
+      <x:c r="L1" s="1"/>
+      <x:c r="M1" s="1"/>
+      <x:c r="N1" s="1"/>
+      <x:c r="O1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="3" t="str">
+        <x:v>متن فعلی سفید است؛ هر تغییری که می‌خواهید در ستون زرد روبه‌روی آن بنویسید</x:v>
+      </x:c>
+      <x:c r="B2" s="3"/>
+      <x:c r="C2" s="3"/>
+      <x:c r="D2" s="3"/>
+      <x:c r="E2" s="3"/>
+      <x:c r="F2" s="3"/>
+      <x:c r="G2" s="3"/>
+      <x:c r="H2" s="3"/>
+      <x:c r="I2" s="3"/>
+      <x:c r="J2" s="3"/>
+      <x:c r="K2" s="3"/>
+      <x:c r="L2" s="3"/>
+      <x:c r="M2" s="3"/>
+      <x:c r="N2" s="3"/>
+      <x:c r="O2" s="3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="20" t="str">
+        <x:v>پیش‌نمایش تصویر</x:v>
+      </x:c>
+      <x:c r="B4" s="20" t="str">
+        <x:v>عنوان فعلی</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>عنوان پیشنهادی شما</x:v>
+      </x:c>
+      <x:c r="D4" s="20" t="str">
+        <x:v>توضیح فعلی</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="str">
+        <x:v>توضیح پیشنهادی شما</x:v>
+      </x:c>
+      <x:c r="F4" s="20" t="str">
+        <x:v>روش بازی فعلی</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="str">
+        <x:v>روش پیشنهادی شما</x:v>
+      </x:c>
+      <x:c r="H4" s="20" t="str">
+        <x:v>نکته ایمنی فعلی</x:v>
+      </x:c>
+      <x:c r="I4" s="21" t="str">
+        <x:v>ایمنی پیشنهادی شما</x:v>
+      </x:c>
+      <x:c r="J4" s="21" t="str">
+        <x:v>تصمیم متن</x:v>
+      </x:c>
+      <x:c r="K4" s="21" t="str">
+        <x:v>تصمیم تصویر</x:v>
+      </x:c>
+      <x:c r="L4" s="21" t="str">
+        <x:v>فایل یا نشانی تصویر</x:v>
+      </x:c>
+      <x:c r="M4" s="21" t="str">
+        <x:v>متن جایگزین تصویر</x:v>
+      </x:c>
+      <x:c r="N4" s="21" t="str">
+        <x:v>نکته برش</x:v>
+      </x:c>
+      <x:c r="O4" s="21" t="str">
+        <x:v>یادداشت شما</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="118" customHeight="1">
+      <x:c r="A5" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B5" s="22" t="str">
+        <x:v>آینه‌ی شکلک‌ها</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str"/>
+      <x:c r="D5" s="22" t="str">
+        <x:v>همراه حالت‌های ساده صورت را نشان می‌دهد و به پاسخ کودک فرصت می‌دهد</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str"/>
+      <x:c r="F5" s="22" t="str">
+        <x:v>روبه‌روی کودک بنشینید | یک حالت ساده مثل لبخند نشان دهید | مکث کنید و پاسخ کودک را تقلید کنید</x:v>
+      </x:c>
+      <x:c r="G5" s="23" t="str"/>
+      <x:c r="H5" s="22" t="str">
+        <x:v>اگر کودک روی برمی‌گرداند یا بی‌قرار می‌شود، بازی را متوقف کنید</x:v>
+      </x:c>
+      <x:c r="I5" s="23" t="str"/>
+      <x:c r="J5" s="23" t="str"/>
+      <x:c r="K5" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L5" s="23" t="str"/>
+      <x:c r="M5" s="23" t="str"/>
+      <x:c r="N5" s="23" t="str"/>
+      <x:c r="O5" s="23" t="str"/>
+    </x:row>
+    <x:row r="6" ht="118" customHeight="1">
+      <x:c r="A6" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B6" s="22" t="str">
+        <x:v>آواز و مکث</x:v>
+      </x:c>
+      <x:c r="C6" s="23" t="str"/>
+      <x:c r="D6" s="22" t="str">
+        <x:v>یک آواز کوتاه با مکث‌های منتظرانه به بازی نوبتی تبدیل می‌شود</x:v>
+      </x:c>
+      <x:c r="E6" s="23" t="str"/>
+      <x:c r="F6" s="22" t="str">
+        <x:v>یک آواز آشنا را آرام بخوانید | در پایان هر بخش مکث کنید | به صدا یا حرکت کودک پاسخ دهید</x:v>
+      </x:c>
+      <x:c r="G6" s="23" t="str"/>
+      <x:c r="H6" s="22" t="str">
+        <x:v>صدا را آرام نگه دارید و با نخستین نشانه ناراحتی مکث کنید</x:v>
+      </x:c>
+      <x:c r="I6" s="23" t="str"/>
+      <x:c r="J6" s="23" t="str"/>
+      <x:c r="K6" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L6" s="23" t="str"/>
+      <x:c r="M6" s="23" t="str"/>
+      <x:c r="N6" s="23" t="str"/>
+      <x:c r="O6" s="23" t="str"/>
+    </x:row>
+    <x:row r="7" ht="118" customHeight="1">
+      <x:c r="A7" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B7" s="22" t="str">
+        <x:v>دنبال دست‌های من</x:v>
+      </x:c>
+      <x:c r="C7" s="23" t="str"/>
+      <x:c r="D7" s="22" t="str">
+        <x:v>حرکت آهسته دست همراه، نگاه و رسیدن کودک را به رفت‌وبرگشت کوتاه تبدیل می‌کند</x:v>
+      </x:c>
+      <x:c r="E7" s="23" t="str"/>
+      <x:c r="F7" s="22" t="str">
+        <x:v>کودک را در وضعیت پایدار قرار دهید | دست را آرام از یک سمت به سمت دیگر ببرید | پس از دنبال‌کردن مکث کنید</x:v>
+      </x:c>
+      <x:c r="G7" s="23" t="str"/>
+      <x:c r="H7" s="22" t="str">
+        <x:v>کودک را برای رسیدن یا چرخیدن مجبور نکنید</x:v>
+      </x:c>
+      <x:c r="I7" s="23" t="str"/>
+      <x:c r="J7" s="23" t="str"/>
+      <x:c r="K7" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L7" s="23" t="str"/>
+      <x:c r="M7" s="23" t="str"/>
+      <x:c r="N7" s="23" t="str"/>
+      <x:c r="O7" s="23" t="str"/>
+    </x:row>
+    <x:row r="8" ht="118" customHeight="1">
+      <x:c r="A8" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>صدا از کجاست</x:v>
+      </x:c>
+      <x:c r="C8" s="23" t="str"/>
+      <x:c r="D8" s="22" t="str">
+        <x:v>صدای آرام همراه از جهت‌های نزدیک، کودک را به پیدا کردن منبع صدا دعوت می‌کند</x:v>
+      </x:c>
+      <x:c r="E8" s="23" t="str"/>
+      <x:c r="F8" s="22" t="str">
+        <x:v>کنار کودک و در میدان دید او بنشینید | نام کودک را آرام از یک سمت بگویید | پس از پیدا کردن صدا جهت را عوض کنید</x:v>
+      </x:c>
+      <x:c r="G8" s="23" t="str"/>
+      <x:c r="H8" s="22" t="str">
+        <x:v>صدا را ناگهانی یا نزدیک گوش کودک تولید نکنید</x:v>
+      </x:c>
+      <x:c r="I8" s="23" t="str"/>
+      <x:c r="J8" s="23" t="str"/>
+      <x:c r="K8" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L8" s="23" t="str"/>
+      <x:c r="M8" s="23" t="str"/>
+      <x:c r="N8" s="23" t="str"/>
+      <x:c r="O8" s="23" t="str"/>
+    </x:row>
+    <x:row r="9" ht="118" customHeight="1">
+      <x:c r="A9" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>تو بگو، من تکرار می‌کنم</x:v>
+      </x:c>
+      <x:c r="C9" s="23" t="str"/>
+      <x:c r="D9" s="22" t="str">
+        <x:v>همراه صداها و حرکت‌های کودک را تقلید می‌کند تا کودک رهبر بازی باشد</x:v>
+      </x:c>
+      <x:c r="E9" s="23" t="str"/>
+      <x:c r="F9" s="22" t="str">
+        <x:v>به حرکت یا صدای کودک توجه کنید | همان را آرام تقلید کنید | مکث کنید تا کودک نوبت بعد را آغاز کند</x:v>
+      </x:c>
+      <x:c r="G9" s="23" t="str"/>
+      <x:c r="H9" s="22" t="str">
+        <x:v>بازی را کوتاه نگه دارید و نشانه‌های خستگی را جدی بگیرید</x:v>
+      </x:c>
+      <x:c r="I9" s="23" t="str"/>
+      <x:c r="J9" s="23" t="str"/>
+      <x:c r="K9" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L9" s="23" t="str"/>
+      <x:c r="M9" s="23" t="str"/>
+      <x:c r="N9" s="23" t="str"/>
+      <x:c r="O9" s="23" t="str"/>
+    </x:row>
+    <x:row r="10" ht="118" customHeight="1">
+      <x:c r="A10" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B10" s="22" t="str">
+        <x:v>برج لیوانی</x:v>
+      </x:c>
+      <x:c r="C10" s="23" t="str"/>
+      <x:c r="D10" s="22" t="str">
+        <x:v>کودک و همراه لیوان‌ها را روی هم می‌چینند و دوباره از نو می‌سازند</x:v>
+      </x:c>
+      <x:c r="E10" s="23" t="str"/>
+      <x:c r="F10" s="22" t="str">
+        <x:v>لیوان‌های سبک را روی زمین بگذارید | نوبتی یک لیوان اضافه کنید | برج را خراب و دوباره بسازید</x:v>
+      </x:c>
+      <x:c r="G10" s="23" t="str"/>
+      <x:c r="H10" s="22" t="str">
+        <x:v>فقط از لیوان سبک و نشکن استفاده کنید</x:v>
+      </x:c>
+      <x:c r="I10" s="23" t="str"/>
+      <x:c r="J10" s="23" t="str"/>
+      <x:c r="K10" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L10" s="23" t="str"/>
+      <x:c r="M10" s="23" t="str"/>
+      <x:c r="N10" s="23" t="str"/>
+      <x:c r="O10" s="23" t="str"/>
+    </x:row>
+    <x:row r="11" ht="118" customHeight="1">
+      <x:c r="A11" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B11" s="22" t="str">
+        <x:v>راه‌رفتن حیوان‌ها</x:v>
+      </x:c>
+      <x:c r="C11" s="23" t="str"/>
+      <x:c r="D11" s="22" t="str">
+        <x:v>کودک و همراه حرکت چند حیوان را آرام و خنده‌دار تقلید می‌کنند</x:v>
+      </x:c>
+      <x:c r="E11" s="23" t="str"/>
+      <x:c r="F11" s="22" t="str">
+        <x:v>یک حیوان با حرکت ساده انتخاب کنید | حرکت را آهسته نشان دهید | نقش انتخاب حیوان را عوض کنید</x:v>
+      </x:c>
+      <x:c r="G11" s="23" t="str"/>
+      <x:c r="H11" s="22" t="str">
+        <x:v>فضا را از لبه و مانع خالی کنید و حرکت‌های پرشی را حذف کنید</x:v>
+      </x:c>
+      <x:c r="I11" s="23" t="str"/>
+      <x:c r="J11" s="23" t="str"/>
+      <x:c r="K11" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L11" s="23" t="str"/>
+      <x:c r="M11" s="23" t="str"/>
+      <x:c r="N11" s="23" t="str"/>
+      <x:c r="O11" s="23" t="str"/>
+    </x:row>
+    <x:row r="12" ht="118" customHeight="1">
+      <x:c r="A12" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>رنگ را پیدا کن</x:v>
+      </x:c>
+      <x:c r="C12" s="23" t="str"/>
+      <x:c r="D12" s="22" t="str">
+        <x:v>همراه یک رنگ می‌گوید و کودک در فضای نزدیک چیزی هم‌رنگ پیدا می‌کند</x:v>
+      </x:c>
+      <x:c r="E12" s="23" t="str"/>
+      <x:c r="F12" s="22" t="str">
+        <x:v>یک رنگ آشنا را نام ببرید | از کودک بخواهید همان رنگ را نشان دهد | پس از پاسخ رنگ بعدی را بگویید</x:v>
+      </x:c>
+      <x:c r="G12" s="23" t="str"/>
+      <x:c r="H12" s="22" t="str">
+        <x:v>فقط اشیای در دسترس را انتخاب کنید و اجازه بالارفتن ندهید</x:v>
+      </x:c>
+      <x:c r="I12" s="23" t="str"/>
+      <x:c r="J12" s="23" t="str"/>
+      <x:c r="K12" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L12" s="23" t="str"/>
+      <x:c r="M12" s="23" t="str"/>
+      <x:c r="N12" s="23" t="str"/>
+      <x:c r="O12" s="23" t="str"/>
+    </x:row>
+    <x:row r="13" ht="118" customHeight="1">
+      <x:c r="A13" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>قصه‌ی نیمه‌کاره</x:v>
+      </x:c>
+      <x:c r="C13" s="23" t="str"/>
+      <x:c r="D13" s="22" t="str">
+        <x:v>همراه یک قصه کوتاه می‌گوید و کودک با صدا یا حرکت ادامه‌اش می‌دهد</x:v>
+      </x:c>
+      <x:c r="E13" s="23" t="str"/>
+      <x:c r="F13" s="22" t="str">
+        <x:v>قصه را با یک شخصیت آشنا شروع کنید | پس از یک جمله مکث کنید | پاسخ کودک را در جمله بعد وارد کنید</x:v>
+      </x:c>
+      <x:c r="G13" s="23" t="str"/>
+      <x:c r="H13" s="22" t="str">
+        <x:v>از صدای ناگهانی و موضوع ترسناک استفاده نکنید</x:v>
+      </x:c>
+      <x:c r="I13" s="23" t="str"/>
+      <x:c r="J13" s="23" t="str"/>
+      <x:c r="K13" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L13" s="23" t="str"/>
+      <x:c r="M13" s="23" t="str"/>
+      <x:c r="N13" s="23" t="str"/>
+      <x:c r="O13" s="23" t="str"/>
+    </x:row>
+    <x:row r="14" ht="118" customHeight="1">
+      <x:c r="A14" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B14" s="22" t="str">
+        <x:v>جورچین لباس‌ها</x:v>
+      </x:c>
+      <x:c r="C14" s="23" t="str"/>
+      <x:c r="D14" s="22" t="str">
+        <x:v>لباس‌های تمیز با رنگ یا اندازه به دسته‌های ساده تقسیم می‌شوند</x:v>
+      </x:c>
+      <x:c r="E14" s="23" t="str"/>
+      <x:c r="F14" s="22" t="str">
+        <x:v>چند لباس تمیز را روی زمین بگذارید | یک قانون ساده انتخاب کنید | با هم دسته‌بندی و جمع کنید</x:v>
+      </x:c>
+      <x:c r="G14" s="23" t="str"/>
+      <x:c r="H14" s="22" t="str">
+        <x:v>کیسه پلاستیکی، بند بلند و قطعه جداشدنی را وارد بازی نکنید</x:v>
+      </x:c>
+      <x:c r="I14" s="23" t="str"/>
+      <x:c r="J14" s="23" t="str"/>
+      <x:c r="K14" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L14" s="23" t="str"/>
+      <x:c r="M14" s="23" t="str"/>
+      <x:c r="N14" s="23" t="str"/>
+      <x:c r="O14" s="23" t="str"/>
+    </x:row>
+    <x:row r="15" ht="118" customHeight="1">
+      <x:c r="A15" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B15" s="22" t="str">
+        <x:v>مجسمه با دست‌زدن</x:v>
+      </x:c>
+      <x:c r="C15" s="23" t="str"/>
+      <x:c r="D15" s="22" t="str">
+        <x:v>کودک با ریتم دست‌زدن حرکت می‌کند و با قطع صدا بی‌حرکت می‌ماند</x:v>
+      </x:c>
+      <x:c r="E15" s="23" t="str"/>
+      <x:c r="F15" s="22" t="str">
+        <x:v>فضای حرکت را خالی کنید | با دست‌زدن آرام ریتم بسازید | مکث کنید و مثل مجسمه بایستید</x:v>
+      </x:c>
+      <x:c r="G15" s="23" t="str"/>
+      <x:c r="H15" s="22" t="str">
+        <x:v>دویدن و پریدن کنار وسایل را حذف کنید</x:v>
+      </x:c>
+      <x:c r="I15" s="23" t="str"/>
+      <x:c r="J15" s="23" t="str"/>
+      <x:c r="K15" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L15" s="23" t="str"/>
+      <x:c r="M15" s="23" t="str"/>
+      <x:c r="N15" s="23" t="str"/>
+      <x:c r="O15" s="23" t="str"/>
+    </x:row>
+    <x:row r="16" ht="118" customHeight="1">
+      <x:c r="A16" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B16" s="22" t="str">
+        <x:v>مسیر پتویی</x:v>
+      </x:c>
+      <x:c r="C16" s="23" t="str"/>
+      <x:c r="D16" s="22" t="str">
+        <x:v>یک پتوی پهن‌شده به مسیر خیالی برای قدم‌های آهسته تبدیل می‌شود</x:v>
+      </x:c>
+      <x:c r="E16" s="23" t="str"/>
+      <x:c r="F16" s="22" t="str">
+        <x:v>پتو را صاف روی سطح بدون لغزش پهن کنید | مسیر را جاده خیالی بنامید | نوبتی روی مسیر قدم بزنید</x:v>
+      </x:c>
+      <x:c r="G16" s="23" t="str"/>
+      <x:c r="H16" s="22" t="str">
+        <x:v>لبه پتو نباید جمع یا لغزنده باشد و دویدن ممنوع است</x:v>
+      </x:c>
+      <x:c r="I16" s="23" t="str"/>
+      <x:c r="J16" s="23" t="str"/>
+      <x:c r="K16" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L16" s="23" t="str"/>
+      <x:c r="M16" s="23" t="str"/>
+      <x:c r="N16" s="23" t="str"/>
+      <x:c r="O16" s="23" t="str"/>
+    </x:row>
+    <x:row r="17" ht="118" customHeight="1">
+      <x:c r="A17" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>زنجیره‌ی نقاشی</x:v>
+      </x:c>
+      <x:c r="C17" s="23" t="str"/>
+      <x:c r="D17" s="22" t="str">
+        <x:v>هر نفر یک خط به نقاشی اضافه می‌کند تا تصویر مشترک شکل بگیرد</x:v>
+      </x:c>
+      <x:c r="E17" s="23" t="str"/>
+      <x:c r="F17" s="22" t="str">
+        <x:v>یک کاغذ آماده کنید | نفر اول یک شکل ساده بکشد | نوبتی یک بخش اضافه کنید</x:v>
+      </x:c>
+      <x:c r="G17" s="23" t="str"/>
+      <x:c r="H17" s="22" t="str">
+        <x:v>از ابزار نقاشی مناسب سن و غیرسمی استفاده کنید</x:v>
+      </x:c>
+      <x:c r="I17" s="23" t="str"/>
+      <x:c r="J17" s="23" t="str"/>
+      <x:c r="K17" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L17" s="23" t="str"/>
+      <x:c r="M17" s="23" t="str"/>
+      <x:c r="N17" s="23" t="str"/>
+      <x:c r="O17" s="23" t="str"/>
+    </x:row>
+    <x:row r="18" ht="118" customHeight="1">
+      <x:c r="A18" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B18" s="22" t="str">
+        <x:v>صدای قصه</x:v>
+      </x:c>
+      <x:c r="C18" s="23" t="str"/>
+      <x:c r="D18" s="22" t="str">
+        <x:v>یک قصه کوتاه با صداهای انتخابی کودک جان می‌گیرد</x:v>
+      </x:c>
+      <x:c r="E18" s="23" t="str"/>
+      <x:c r="F18" s="22" t="str">
+        <x:v>یک قصه ساده شروع کنید | برای دو اتفاق صدای کوتاه انتخاب کنید | در قصه مکث کنید تا کودک صدا را بسازد</x:v>
+      </x:c>
+      <x:c r="G18" s="23" t="str"/>
+      <x:c r="H18" s="22" t="str">
+        <x:v>صداها را ملایم نگه دارید و با ناراحتی کودک موضوع را عوض کنید</x:v>
+      </x:c>
+      <x:c r="I18" s="23" t="str"/>
+      <x:c r="J18" s="23" t="str"/>
+      <x:c r="K18" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L18" s="23" t="str"/>
+      <x:c r="M18" s="23" t="str"/>
+      <x:c r="N18" s="23" t="str"/>
+      <x:c r="O18" s="23" t="str"/>
+    </x:row>
+    <x:row r="19" ht="118" customHeight="1">
+      <x:c r="A19" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>دروازه‌ی توپ نرم</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="str"/>
+      <x:c r="D19" s="22" t="str">
+        <x:v>توپ نرم نوبتی از میان یک دروازه خیالی به سمت هم قل داده می‌شود</x:v>
+      </x:c>
+      <x:c r="E19" s="23" t="str"/>
+      <x:c r="F19" s="22" t="str">
+        <x:v>دو نشانه امن برای دروازه بگذارید | روبه‌روی هم روی زمین بنشینید | توپ را نوبتی از دروازه قل دهید</x:v>
+      </x:c>
+      <x:c r="G19" s="23" t="str"/>
+      <x:c r="H19" s="22" t="str">
+        <x:v>فقط توپ نرم استفاده شود و توپ پرتاب نشود</x:v>
+      </x:c>
+      <x:c r="I19" s="23" t="str"/>
+      <x:c r="J19" s="23" t="str"/>
+      <x:c r="K19" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L19" s="23" t="str"/>
+      <x:c r="M19" s="23" t="str"/>
+      <x:c r="N19" s="23" t="str"/>
+      <x:c r="O19" s="23" t="str"/>
+    </x:row>
+    <x:row r="20" ht="118" customHeight="1">
+      <x:c r="A20" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B20" s="22" t="str">
+        <x:v>نقشه‌ی گنج کاغذی</x:v>
+      </x:c>
+      <x:c r="C20" s="23" t="str"/>
+      <x:c r="D20" s="22" t="str">
+        <x:v>کودک و همراه نقشه‌ای ساده می‌کشند و یک مقصد خیالی پیدا می‌کنند</x:v>
+      </x:c>
+      <x:c r="E20" s="23" t="str"/>
+      <x:c r="F20" s="22" t="str">
+        <x:v>سه نقطه آشنا را روی کاغذ علامت بزنید | یک مسیر ساده بکشید | با هم مسیر را طی کنید</x:v>
+      </x:c>
+      <x:c r="G20" s="23" t="str"/>
+      <x:c r="H20" s="22" t="str">
+        <x:v>مسیر نباید از پله، بالارفتن یا محل خطرناک عبور کند</x:v>
+      </x:c>
+      <x:c r="I20" s="23" t="str"/>
+      <x:c r="J20" s="23" t="str"/>
+      <x:c r="K20" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L20" s="23" t="str"/>
+      <x:c r="M20" s="23" t="str"/>
+      <x:c r="N20" s="23" t="str"/>
+      <x:c r="O20" s="23" t="str"/>
+    </x:row>
+    <x:row r="21" ht="118" customHeight="1">
+      <x:c r="A21" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B21" s="22" t="str">
+        <x:v>پانتومیم بی‌صدا</x:v>
+      </x:c>
+      <x:c r="C21" s="23" t="str"/>
+      <x:c r="D21" s="22" t="str">
+        <x:v>هر نفر یک کار روزمره را بی‌صدا اجرا می‌کند و دیگری حدس می‌زند</x:v>
+      </x:c>
+      <x:c r="E21" s="23" t="str"/>
+      <x:c r="F21" s="22" t="str">
+        <x:v>یک کار ساده انتخاب کنید | بدون حرف‌زدن آن را نشان دهید | پس از حدس نقش‌ها را عوض کنید</x:v>
+      </x:c>
+      <x:c r="G21" s="23" t="str"/>
+      <x:c r="H21" s="22" t="str">
+        <x:v>حرکت‌ها بدون دویدن، پرتاب یا تقلید کار خطرناک باشند</x:v>
+      </x:c>
+      <x:c r="I21" s="23" t="str"/>
+      <x:c r="J21" s="23" t="str"/>
+      <x:c r="K21" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L21" s="23" t="str"/>
+      <x:c r="M21" s="23" t="str"/>
+      <x:c r="N21" s="23" t="str"/>
+      <x:c r="O21" s="23" t="str"/>
+    </x:row>
+    <x:row r="22" ht="118" customHeight="1">
+      <x:c r="A22" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B22" s="22" t="str">
+        <x:v>چالش برج کاغذی</x:v>
+      </x:c>
+      <x:c r="C22" s="23" t="str"/>
+      <x:c r="D22" s="22" t="str">
+        <x:v>با چند برگ کاغذ و بدون چسب، یک سازه ایستاده ساخته می‌شود</x:v>
+      </x:c>
+      <x:c r="E22" s="23" t="str"/>
+      <x:c r="F22" s="22" t="str">
+        <x:v>کاغذها را روی سطح صاف بگذارید | با تا کردن قطعه بسازید | نوبتی قطعه اضافه کنید</x:v>
+      </x:c>
+      <x:c r="G22" s="23" t="str"/>
+      <x:c r="H22" s="22" t="str">
+        <x:v>کاغذ را نزدیک صورت پرتاب نکنید و تکه‌ها را جمع کنید</x:v>
+      </x:c>
+      <x:c r="I22" s="23" t="str"/>
+      <x:c r="J22" s="23" t="str"/>
+      <x:c r="K22" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L22" s="23" t="str"/>
+      <x:c r="M22" s="23" t="str"/>
+      <x:c r="N22" s="23" t="str"/>
+      <x:c r="O22" s="23" t="str"/>
+    </x:row>
+    <x:row r="23" ht="118" customHeight="1">
+      <x:c r="A23" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B23" s="22" t="str">
+        <x:v>داستان زنجیره‌ای</x:v>
+      </x:c>
+      <x:c r="C23" s="23" t="str"/>
+      <x:c r="D23" s="22" t="str">
+        <x:v>هر نفر فقط یک جمله به داستان مشترک اضافه می‌کند</x:v>
+      </x:c>
+      <x:c r="E23" s="23" t="str"/>
+      <x:c r="F23" s="22" t="str">
+        <x:v>نفر اول شخصیت و مکان را معرفی کند | نفر بعد یک جمله ادامه دهد | پس از سه دور داستان را تمام کنید</x:v>
+      </x:c>
+      <x:c r="G23" s="23" t="str"/>
+      <x:c r="H23" s="22" t="str">
+        <x:v>از موضوع ترسناک یا ناراحت‌کننده دوری کنید</x:v>
+      </x:c>
+      <x:c r="I23" s="23" t="str"/>
+      <x:c r="J23" s="23" t="str"/>
+      <x:c r="K23" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L23" s="23" t="str"/>
+      <x:c r="M23" s="23" t="str"/>
+      <x:c r="N23" s="23" t="str"/>
+      <x:c r="O23" s="23" t="str"/>
+    </x:row>
+    <x:row r="24" ht="118" customHeight="1">
+      <x:c r="A24" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B24" s="22" t="str">
+        <x:v>هدف‌گیری با توپ نرم</x:v>
+      </x:c>
+      <x:c r="C24" s="23" t="str"/>
+      <x:c r="D24" s="22" t="str">
+        <x:v>بازیکن‌ها توپ نرم را به محدوده‌ای روی زمین هدایت می‌کنند و امتیاز گروهی می‌سازند</x:v>
+      </x:c>
+      <x:c r="E24" s="23" t="str"/>
+      <x:c r="F24" s="22" t="str">
+        <x:v>یک محدوده امن تعیین کنید | از فاصله کوتاه توپ را قل دهید | امتیازها را برای رکورد مشترک جمع کنید</x:v>
+      </x:c>
+      <x:c r="G24" s="23" t="str"/>
+      <x:c r="H24" s="22" t="str">
+        <x:v>توپ فقط روی زمین قل داده شود و اطراف خالی باشد</x:v>
+      </x:c>
+      <x:c r="I24" s="23" t="str"/>
+      <x:c r="J24" s="23" t="str"/>
+      <x:c r="K24" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L24" s="23" t="str"/>
+      <x:c r="M24" s="23" t="str"/>
+      <x:c r="N24" s="23" t="str"/>
+      <x:c r="O24" s="23" t="str"/>
+    </x:row>
+    <x:row r="25" ht="118" customHeight="1">
+      <x:c r="A25" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B25" s="22" t="str">
+        <x:v>بیست سؤال خانوادگی</x:v>
+      </x:c>
+      <x:c r="C25" s="23" t="str"/>
+      <x:c r="D25" s="22" t="str">
+        <x:v>یک نفر چیزی را در ذهن نگه می‌دارد و دیگران با سؤال‌های بله یا خیر آن را پیدا می‌کنند</x:v>
+      </x:c>
+      <x:c r="E25" s="23" t="str"/>
+      <x:c r="F25" s="22" t="str">
+        <x:v>یک موضوع آشنا انتخاب کنید | فقط سؤال بله یا خیر بپرسید | پس از حدس انتخاب‌کننده را عوض کنید</x:v>
+      </x:c>
+      <x:c r="G25" s="23" t="str"/>
+      <x:c r="H25" s="22" t="str">
+        <x:v>موضوع‌ها را محترمانه و غیرشخصی نگه دارید</x:v>
+      </x:c>
+      <x:c r="I25" s="23" t="str"/>
+      <x:c r="J25" s="23" t="str"/>
+      <x:c r="K25" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L25" s="23" t="str"/>
+      <x:c r="M25" s="23" t="str"/>
+      <x:c r="N25" s="23" t="str"/>
+      <x:c r="O25" s="23" t="str"/>
+    </x:row>
+    <x:row r="26" ht="118" customHeight="1">
+      <x:c r="A26" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B26" s="22" t="str">
+        <x:v>مأموریت بی‌صدا</x:v>
+      </x:c>
+      <x:c r="C26" s="23" t="str"/>
+      <x:c r="D26" s="22" t="str">
+        <x:v>گروه باید یک کار ساده را بدون حرف‌زدن و فقط با اشاره هماهنگ کند</x:v>
+      </x:c>
+      <x:c r="E26" s="23" t="str"/>
+      <x:c r="F26" s="22" t="str">
+        <x:v>یک مأموریت امن انتخاب کنید | تا پایان مأموریت حرف نزنید | درباره اشاره‌های مؤثر گفت‌وگو کنید</x:v>
+      </x:c>
+      <x:c r="G26" s="23" t="str"/>
+      <x:c r="H26" s="22" t="str">
+        <x:v>مأموریت شامل دویدن، بالارفتن یا وسیله سنگین نباشد</x:v>
+      </x:c>
+      <x:c r="I26" s="23" t="str"/>
+      <x:c r="J26" s="23" t="str"/>
+      <x:c r="K26" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L26" s="23" t="str"/>
+      <x:c r="M26" s="23" t="str"/>
+      <x:c r="N26" s="23" t="str"/>
+      <x:c r="O26" s="23" t="str"/>
+    </x:row>
+    <x:row r="27" ht="118" customHeight="1">
+      <x:c r="A27" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B27" s="22" t="str">
+        <x:v>بازی کاغذی خودمان</x:v>
+      </x:c>
+      <x:c r="C27" s="23" t="str"/>
+      <x:c r="D27" s="22" t="str">
+        <x:v>کودک و همراه با چند قانون ساده یک بازی رومیزی کوچک طراحی می‌کنند</x:v>
+      </x:c>
+      <x:c r="E27" s="23" t="str"/>
+      <x:c r="F27" s="22" t="str">
+        <x:v>هدف بازی را در یک جمله بنویسید | سه قانون کوتاه تعیین کنید | یک دور آزمایشی اجرا و یک قانون را بهتر کنید</x:v>
+      </x:c>
+      <x:c r="G27" s="23" t="str"/>
+      <x:c r="H27" s="22" t="str">
+        <x:v>از مهره ریز، ابزار برنده و قانون تنبیهی استفاده نکنید</x:v>
+      </x:c>
+      <x:c r="I27" s="23" t="str"/>
+      <x:c r="J27" s="23" t="str"/>
+      <x:c r="K27" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L27" s="23" t="str"/>
+      <x:c r="M27" s="23" t="str"/>
+      <x:c r="N27" s="23" t="str"/>
+      <x:c r="O27" s="23" t="str"/>
+    </x:row>
+    <x:row r="28" ht="118" customHeight="1">
+      <x:c r="A28" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B28" s="22" t="str">
+        <x:v>مناظره‌ی خنده‌دار</x:v>
+      </x:c>
+      <x:c r="C28" s="23" t="str"/>
+      <x:c r="D28" s="22" t="str">
+        <x:v>دو طرف از انتخاب‌های بی‌خطر و خیالی دفاع می‌کنند و سپس جای‌شان را عوض می‌کنند</x:v>
+      </x:c>
+      <x:c r="E28" s="23" t="str"/>
+      <x:c r="F28" s="22" t="str">
+        <x:v>یک موضوع سبک انتخاب کنید | هر نفر یک دقیقه دلیل بگوید | نقش‌ها را عوض کنید</x:v>
+      </x:c>
+      <x:c r="G28" s="23" t="str"/>
+      <x:c r="H28" s="22" t="str">
+        <x:v>موضوع درباره ظاهر، هویت یا نقطه‌ضعف افراد نباشد</x:v>
+      </x:c>
+      <x:c r="I28" s="23" t="str"/>
+      <x:c r="J28" s="23" t="str"/>
+      <x:c r="K28" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L28" s="23" t="str"/>
+      <x:c r="M28" s="23" t="str"/>
+      <x:c r="N28" s="23" t="str"/>
+      <x:c r="O28" s="23" t="str"/>
+    </x:row>
+    <x:row r="29" ht="118" customHeight="1">
+      <x:c r="A29" s="22" t="str">
+        <x:v>هنوز تصویر پیشنهادی نداریم</x:v>
+      </x:c>
+      <x:c r="B29" s="22" t="str">
+        <x:v>پل کاغذی</x:v>
+      </x:c>
+      <x:c r="C29" s="23" t="str"/>
+      <x:c r="D29" s="22" t="str">
+        <x:v>گروه با تا کردن کاغذ پلی می‌سازد که یک لیوان خالی را نگه دارد</x:v>
+      </x:c>
+      <x:c r="E29" s="23" t="str"/>
+      <x:c r="F29" s="22" t="str">
+        <x:v>دو تکیه‌گاه سبک آماده کنید | کاغذ را تا کنید و میان آن‌ها بگذارید | با یک لیوان خالی پل را آزمایش کنید</x:v>
+      </x:c>
+      <x:c r="G29" s="23" t="str"/>
+      <x:c r="H29" s="22" t="str">
+        <x:v>فقط لیوان خالی و سبک استفاده شود و جسم شیشه‌ای وارد بازی نشود</x:v>
+      </x:c>
+      <x:c r="I29" s="23" t="str"/>
+      <x:c r="J29" s="23" t="str"/>
+      <x:c r="K29" s="23" t="str">
+        <x:v>در انتظار تصویر</x:v>
+      </x:c>
+      <x:c r="L29" s="23" t="str"/>
+      <x:c r="M29" s="23" t="str"/>
+      <x:c r="N29" s="23" t="str"/>
+      <x:c r="O29" s="23" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="J5:J29">
+      <x:formula1>"تأیید,نیاز به اصلاح,رد"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K5:K29">
+      <x:formula1>"در انتظار تصویر,در انتظار بررسی,تأیید,نیاز به اصلاح,رد"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fcbe6015f1c4b29"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -3684,12 +4621,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R962d8c5b967b4fbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2793d5b795d4495"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4415,12 +5352,12 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re01bfea7cbbb4b23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77e081f412dc4c4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -4798,7 +5735,79 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf2e3ca6da184092"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf23f1a82c804f0c"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>مرجع سبک تصویر بازی‌ها</x:v>
+      </x:c>
+      <x:c r="B1" s="1"/>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="1"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
+      <x:c r="I1" s="1"/>
+      <x:c r="J1" s="1"/>
+      <x:c r="K1" s="1"/>
+      <x:c r="L1" s="1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="3" t="str">
+        <x:v>این تصویر فقط سبک موردنظر را نشان می‌دهد و کاور نهایی هیچ‌کدام از ۲۵ بازی نیست</x:v>
+      </x:c>
+      <x:c r="B2" s="3"/>
+      <x:c r="C2" s="3"/>
+      <x:c r="D2" s="3"/>
+      <x:c r="E2" s="3"/>
+      <x:c r="F2" s="3"/>
+      <x:c r="G2" s="3"/>
+      <x:c r="H2" s="3"/>
+      <x:c r="I2" s="3"/>
+      <x:c r="J2" s="3"/>
+      <x:c r="K2" s="3"/>
+      <x:c r="L2" s="3"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="29" t="str">
+        <x:v>رنگ گرم، شیء اصلی بازی، بافت نرم و یک تیله واقعی در قاب؛ بدون نوشته داخل تصویر</x:v>
+      </x:c>
+      <x:c r="B3" s="29"/>
+      <x:c r="C3" s="29"/>
+      <x:c r="D3" s="29"/>
+      <x:c r="E3" s="29"/>
+      <x:c r="F3" s="29"/>
+      <x:c r="G3" s="29"/>
+      <x:c r="H3" s="29"/>
+      <x:c r="I3" s="29"/>
+      <x:c r="J3" s="29"/>
+      <x:c r="K3" s="29"/>
+      <x:c r="L3" s="29"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8bf07030868444f"/>
+</x:worksheet>
 </file>
</xml_diff>